<commit_message>
ajustes buscador y layout
</commit_message>
<xml_diff>
--- a/piloto_datos_minerva.xlsx
+++ b/piloto_datos_minerva.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29825"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://agenciadeaduanapirazzoli-my.sharepoint.com/personal/pablo_pirazzoli_cl/Documents/AA_PIRAZZOLI/Proyectos/PROVISORIO_MINERVA/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ale\zz_ale_cosas\otras_personas\Pirazzoli\pirazzoli-demo\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{C39F16CA-2C40-4AC2-AC37-DCF0E665585B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="2" activeTab="2" xr2:uid="{7618C72B-C967-4346-827E-EFA46EAC6289}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" xr2:uid="{7618C72B-C967-4346-827E-EFA46EAC6289}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -1420,7 +1420,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="21">
     <font>
@@ -2007,8 +2007,8 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2024,18 +2024,18 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="43" fontId="4" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2047,7 +2047,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2061,7 +2061,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="43" fontId="4" fillId="3" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2163,9 +2163,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2348,10 +2348,10 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="43" fontId="4" fillId="6" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="6" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="43" fontId="4" fillId="6" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="6" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2388,8 +2388,8 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="3" fillId="8" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="3" fillId="8" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="8" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="8" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2398,8 +2398,8 @@
     <xf numFmtId="22" fontId="0" fillId="8" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="43" fontId="0" fillId="8" borderId="17" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="0" fillId="8" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="17" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="22" fontId="3" fillId="8" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2712,12 +2712,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="16" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2732,6 +2726,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2752,9 +2752,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2792,7 +2792,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2898,7 +2898,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -3040,7 +3040,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -3049,7 +3049,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4B03264-199A-4886-857D-303C27604CC4}">
   <dimension ref="A1:AN225"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.5703125" customWidth="1"/>
     <col min="2" max="2" width="9.140625"/>
@@ -3169,7 +3169,7 @@
       <c r="AL2" s="14"/>
       <c r="AM2" s="14"/>
     </row>
-    <row r="3" spans="1:40" ht="198">
+    <row r="3" spans="1:40" ht="195">
       <c r="B3" s="8" t="s">
         <v>0</v>
       </c>
@@ -3220,7 +3220,7 @@
       </c>
       <c r="AM3" s="106"/>
     </row>
-    <row r="4" spans="1:40" ht="60.75">
+    <row r="4" spans="1:40" ht="60">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -3479,7 +3479,7 @@
       <c r="O6" s="96">
         <v>2605101385</v>
       </c>
-      <c r="P6" s="315">
+      <c r="P6" s="313">
         <v>2605109992</v>
       </c>
       <c r="Q6" s="101" t="s">
@@ -3649,7 +3649,7 @@
       <c r="O8" s="96">
         <v>260595504</v>
       </c>
-      <c r="P8" s="315">
+      <c r="P8" s="313">
         <v>260597318</v>
       </c>
       <c r="Q8" s="101" t="s">
@@ -3815,7 +3815,7 @@
       <c r="O10" s="96">
         <v>2605101685</v>
       </c>
-      <c r="P10" s="315">
+      <c r="P10" s="313">
         <v>2605107573</v>
       </c>
       <c r="Q10" s="101" t="s">
@@ -3897,7 +3897,7 @@
       <c r="O11" s="96">
         <v>2605101914</v>
       </c>
-      <c r="P11" s="315">
+      <c r="P11" s="313">
         <v>2605102768</v>
       </c>
       <c r="Q11" s="101" t="s">
@@ -3979,7 +3979,7 @@
       <c r="O12" s="96">
         <v>2605100691</v>
       </c>
-      <c r="P12" s="315">
+      <c r="P12" s="313">
         <v>2605101997</v>
       </c>
       <c r="Q12" s="101" t="s">
@@ -4065,7 +4065,7 @@
       <c r="O13" s="96">
         <v>2605101437</v>
       </c>
-      <c r="P13" s="315">
+      <c r="P13" s="313">
         <v>2605101999</v>
       </c>
       <c r="Q13" s="101" t="s">
@@ -4147,7 +4147,7 @@
       <c r="O14" s="96">
         <v>2605106858</v>
       </c>
-      <c r="P14" s="315">
+      <c r="P14" s="313">
         <v>2605107743</v>
       </c>
       <c r="Q14" s="101" t="s">
@@ -4219,7 +4219,7 @@
       <c r="O15" s="96">
         <v>2605100503</v>
       </c>
-      <c r="P15" s="315">
+      <c r="P15" s="313">
         <v>2605102001</v>
       </c>
       <c r="Q15" s="101" t="s">
@@ -4295,7 +4295,7 @@
       <c r="O16" s="96">
         <v>2605106749</v>
       </c>
-      <c r="P16" s="315">
+      <c r="P16" s="313">
         <v>2605107710</v>
       </c>
       <c r="Q16" s="101" t="s">
@@ -4377,7 +4377,7 @@
       <c r="O17" s="96">
         <v>2605104506</v>
       </c>
-      <c r="P17" s="315">
+      <c r="P17" s="313">
         <v>2605105058</v>
       </c>
       <c r="Q17" s="101" t="s">
@@ -4627,7 +4627,7 @@
       <c r="O20" s="96">
         <v>2605102035</v>
       </c>
-      <c r="P20" s="315">
+      <c r="P20" s="313">
         <v>2605102626</v>
       </c>
       <c r="Q20" s="101" t="s">
@@ -4707,7 +4707,7 @@
       <c r="O21" s="96">
         <v>2605103273</v>
       </c>
-      <c r="P21" s="315">
+      <c r="P21" s="313">
         <v>2605104792</v>
       </c>
       <c r="Q21" s="101" t="s">
@@ -4787,7 +4787,7 @@
       <c r="O22" s="96">
         <v>2605107269</v>
       </c>
-      <c r="P22" s="315">
+      <c r="P22" s="313">
         <v>2605110378</v>
       </c>
       <c r="Q22" s="100" t="s">
@@ -4868,7 +4868,7 @@
       <c r="O23" s="96">
         <v>2605107217</v>
       </c>
-      <c r="P23" s="315">
+      <c r="P23" s="313">
         <v>2605110317</v>
       </c>
       <c r="Q23" s="64" t="s">
@@ -4948,7 +4948,7 @@
       <c r="O24" s="67">
         <v>2605107322</v>
       </c>
-      <c r="P24" s="315">
+      <c r="P24" s="313">
         <v>2605110277</v>
       </c>
       <c r="Q24" s="100" t="s">
@@ -4979,7 +4979,7 @@
       <c r="AF24" s="118">
         <v>46088.412118055552</v>
       </c>
-      <c r="AG24" s="316" t="s">
+      <c r="AG24" s="314" t="s">
         <v>82</v>
       </c>
       <c r="AH24" s="80"/>
@@ -5008,8 +5008,8 @@
       <c r="G25" s="7" t="s">
         <v>173</v>
       </c>
-      <c r="H25" s="315"/>
-      <c r="I25" s="317"/>
+      <c r="H25" s="313"/>
+      <c r="I25" s="315"/>
       <c r="J25" s="31"/>
       <c r="K25" s="6"/>
       <c r="L25" s="7" t="s">
@@ -5022,7 +5022,7 @@
       <c r="O25" s="97">
         <v>2605103977</v>
       </c>
-      <c r="P25" s="315">
+      <c r="P25" s="313">
         <v>2605104765</v>
       </c>
       <c r="Q25" s="102" t="s">
@@ -5044,10 +5044,10 @@
       <c r="AA25" s="6"/>
       <c r="AB25" s="6"/>
       <c r="AC25" s="24"/>
-      <c r="AD25" s="315"/>
-      <c r="AE25" s="315"/>
-      <c r="AF25" s="315"/>
-      <c r="AG25" s="316"/>
+      <c r="AD25" s="313"/>
+      <c r="AE25" s="313"/>
+      <c r="AF25" s="313"/>
+      <c r="AG25" s="314"/>
       <c r="AH25" s="80"/>
       <c r="AI25" s="80"/>
       <c r="AL25" s="25">
@@ -5092,7 +5092,7 @@
       <c r="O26" s="67">
         <v>2605108712</v>
       </c>
-      <c r="P26" s="315">
+      <c r="P26" s="313">
         <v>2605110144</v>
       </c>
       <c r="Q26" s="101" t="s">
@@ -5116,8 +5116,8 @@
       <c r="AC26" s="24"/>
       <c r="AD26" s="39"/>
       <c r="AE26" s="39"/>
-      <c r="AF26" s="315"/>
-      <c r="AG26" s="316"/>
+      <c r="AF26" s="313"/>
+      <c r="AG26" s="314"/>
       <c r="AH26" s="80"/>
       <c r="AI26" s="80"/>
       <c r="AL26" s="25">
@@ -5162,7 +5162,7 @@
       <c r="O27" s="67">
         <v>2605109923</v>
       </c>
-      <c r="P27" s="315">
+      <c r="P27" s="313">
         <v>2605112548</v>
       </c>
       <c r="Q27" s="101" t="s">
@@ -5322,7 +5322,7 @@
       <c r="O29" s="96">
         <v>2605109152</v>
       </c>
-      <c r="P29" s="315">
+      <c r="P29" s="313">
         <v>2605110090</v>
       </c>
       <c r="Q29" s="100" t="s">
@@ -5345,8 +5345,8 @@
       <c r="AB29" s="6"/>
       <c r="AC29" s="24"/>
       <c r="AD29" s="39"/>
-      <c r="AE29" s="315"/>
-      <c r="AF29" s="315"/>
+      <c r="AE29" s="313"/>
+      <c r="AF29" s="313"/>
       <c r="AG29" s="134"/>
       <c r="AH29" s="81"/>
       <c r="AI29" s="81"/>
@@ -5392,7 +5392,7 @@
       <c r="O30" s="96">
         <v>2605109255</v>
       </c>
-      <c r="P30" s="315">
+      <c r="P30" s="313">
         <v>2605110037</v>
       </c>
       <c r="Q30" s="100" t="s">
@@ -5471,7 +5471,7 @@
       <c r="O31" s="96">
         <v>2605109265</v>
       </c>
-      <c r="P31" s="315">
+      <c r="P31" s="313">
         <v>2605110562</v>
       </c>
       <c r="Q31" s="101" t="s">
@@ -5551,7 +5551,7 @@
       <c r="O32" s="67">
         <v>2605105649</v>
       </c>
-      <c r="P32" s="315">
+      <c r="P32" s="313">
         <v>2605107389</v>
       </c>
       <c r="Q32" s="100" t="s">
@@ -5581,7 +5581,7 @@
       <c r="AE32" s="116">
         <v>46085.672048611108</v>
       </c>
-      <c r="AF32" s="315" t="s">
+      <c r="AF32" s="313" t="s">
         <v>62</v>
       </c>
       <c r="AG32" s="117" t="s">
@@ -5616,7 +5616,7 @@
       <c r="H33" s="39" t="s">
         <v>213</v>
       </c>
-      <c r="I33" s="317" t="s">
+      <c r="I33" s="315" t="s">
         <v>214</v>
       </c>
       <c r="J33" s="31"/>
@@ -5631,7 +5631,7 @@
       <c r="O33" s="67">
         <v>2605109941</v>
       </c>
-      <c r="P33" s="315">
+      <c r="P33" s="313">
         <v>2605112533</v>
       </c>
       <c r="Q33" s="100" t="s">
@@ -5654,9 +5654,9 @@
       <c r="AB33" s="6"/>
       <c r="AC33" s="24"/>
       <c r="AD33" s="39"/>
-      <c r="AE33" s="315"/>
-      <c r="AF33" s="315"/>
-      <c r="AG33" s="316"/>
+      <c r="AE33" s="313"/>
+      <c r="AF33" s="313"/>
+      <c r="AG33" s="314"/>
       <c r="AH33" s="80"/>
       <c r="AI33" s="80"/>
       <c r="AL33" s="25">
@@ -5701,7 +5701,7 @@
       <c r="O34" s="67">
         <v>2605105906</v>
       </c>
-      <c r="P34" s="315">
+      <c r="P34" s="313">
         <v>2605107383</v>
       </c>
       <c r="Q34" s="100" t="s">
@@ -5761,10 +5761,10 @@
       <c r="G35" s="7" t="s">
         <v>222</v>
       </c>
-      <c r="H35" s="315" t="s">
+      <c r="H35" s="313" t="s">
         <v>223</v>
       </c>
-      <c r="I35" s="317" t="s">
+      <c r="I35" s="315" t="s">
         <v>224</v>
       </c>
       <c r="J35" s="31"/>
@@ -5779,7 +5779,7 @@
       <c r="O35" s="67">
         <v>2605109424</v>
       </c>
-      <c r="P35" s="315">
+      <c r="P35" s="313">
         <v>2605110377</v>
       </c>
       <c r="Q35" s="100" t="s">
@@ -5830,10 +5830,10 @@
       <c r="G36" s="7" t="s">
         <v>227</v>
       </c>
-      <c r="H36" s="315" t="s">
+      <c r="H36" s="313" t="s">
         <v>228</v>
       </c>
-      <c r="I36" s="317" t="s">
+      <c r="I36" s="315" t="s">
         <v>229</v>
       </c>
       <c r="J36" s="31"/>
@@ -5848,7 +5848,7 @@
       <c r="O36" s="67">
         <v>2605111544</v>
       </c>
-      <c r="P36" s="315">
+      <c r="P36" s="313">
         <v>2605112433</v>
       </c>
       <c r="Q36" s="100" t="s">
@@ -5860,7 +5860,7 @@
       <c r="T36" s="244">
         <v>4090180178</v>
       </c>
-      <c r="U36" s="317"/>
+      <c r="U36" s="315"/>
       <c r="V36" s="31"/>
       <c r="W36" s="6"/>
       <c r="X36" s="6"/>
@@ -5869,10 +5869,10 @@
       <c r="AA36" s="6"/>
       <c r="AB36" s="6"/>
       <c r="AC36" s="24"/>
-      <c r="AD36" s="315"/>
-      <c r="AE36" s="315"/>
-      <c r="AF36" s="315"/>
-      <c r="AG36" s="316"/>
+      <c r="AD36" s="313"/>
+      <c r="AE36" s="313"/>
+      <c r="AF36" s="313"/>
+      <c r="AG36" s="314"/>
       <c r="AH36" s="80"/>
       <c r="AI36" s="80"/>
       <c r="AL36" s="25"/>
@@ -5897,10 +5897,10 @@
       <c r="G37" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="H37" s="315" t="s">
+      <c r="H37" s="313" t="s">
         <v>233</v>
       </c>
-      <c r="I37" s="317" t="s">
+      <c r="I37" s="315" t="s">
         <v>234</v>
       </c>
       <c r="J37" s="31"/>
@@ -5915,7 +5915,7 @@
       <c r="O37" s="96">
         <v>2605108064</v>
       </c>
-      <c r="P37" s="315">
+      <c r="P37" s="313">
         <v>2605109863</v>
       </c>
       <c r="Q37" s="100" t="s">
@@ -5936,10 +5936,10 @@
       <c r="AA37" s="6"/>
       <c r="AB37" s="6"/>
       <c r="AC37" s="24"/>
-      <c r="AD37" s="315"/>
-      <c r="AE37" s="315"/>
-      <c r="AF37" s="315"/>
-      <c r="AG37" s="316"/>
+      <c r="AD37" s="313"/>
+      <c r="AE37" s="313"/>
+      <c r="AF37" s="313"/>
+      <c r="AG37" s="314"/>
       <c r="AH37" s="80"/>
       <c r="AI37" s="80"/>
       <c r="AL37" s="25"/>
@@ -5982,7 +5982,7 @@
       <c r="O38" s="67">
         <v>2605109685</v>
       </c>
-      <c r="P38" s="315">
+      <c r="P38" s="313">
         <v>2605110139</v>
       </c>
       <c r="Q38" s="100" t="s">
@@ -6004,10 +6004,10 @@
       <c r="AA38" s="6"/>
       <c r="AB38" s="6"/>
       <c r="AC38" s="24"/>
-      <c r="AD38" s="315"/>
-      <c r="AE38" s="315"/>
-      <c r="AF38" s="315"/>
-      <c r="AG38" s="316"/>
+      <c r="AD38" s="313"/>
+      <c r="AE38" s="313"/>
+      <c r="AF38" s="313"/>
+      <c r="AG38" s="314"/>
       <c r="AH38" s="80"/>
       <c r="AI38" s="80"/>
       <c r="AL38" s="25"/>
@@ -6050,7 +6050,7 @@
       <c r="O39" s="97">
         <v>2605109639</v>
       </c>
-      <c r="P39" s="315">
+      <c r="P39" s="313">
         <v>2605110120</v>
       </c>
       <c r="Q39" s="102" t="s">
@@ -6062,7 +6062,7 @@
       <c r="T39" s="244">
         <v>4090180183</v>
       </c>
-      <c r="U39" s="317"/>
+      <c r="U39" s="315"/>
       <c r="V39" s="31"/>
       <c r="W39" s="6"/>
       <c r="X39" s="6"/>
@@ -6071,10 +6071,10 @@
       <c r="AA39" s="6"/>
       <c r="AB39" s="6"/>
       <c r="AC39" s="24"/>
-      <c r="AD39" s="315"/>
-      <c r="AE39" s="315"/>
-      <c r="AF39" s="315"/>
-      <c r="AG39" s="316"/>
+      <c r="AD39" s="313"/>
+      <c r="AE39" s="313"/>
+      <c r="AF39" s="313"/>
+      <c r="AG39" s="314"/>
       <c r="AH39" s="80"/>
       <c r="AI39" s="80"/>
       <c r="AL39" s="25"/>
@@ -6117,7 +6117,7 @@
       <c r="O40" s="67">
         <v>2605111953</v>
       </c>
-      <c r="P40" s="315">
+      <c r="P40" s="313">
         <v>2605112430</v>
       </c>
       <c r="Q40" s="100" t="s">
@@ -6141,7 +6141,7 @@
       <c r="AC40" s="24"/>
       <c r="AD40" s="39"/>
       <c r="AE40" s="39"/>
-      <c r="AF40" s="315"/>
+      <c r="AF40" s="313"/>
       <c r="AG40" s="98"/>
       <c r="AH40" s="80"/>
       <c r="AI40" s="80"/>
@@ -6185,7 +6185,7 @@
       <c r="O41" s="67">
         <v>2605110760</v>
       </c>
-      <c r="P41" s="315">
+      <c r="P41" s="313">
         <v>2605112514</v>
       </c>
       <c r="Q41" s="100" t="s">
@@ -6215,7 +6215,7 @@
       <c r="AE41" s="49">
         <v>46087.774513888886</v>
       </c>
-      <c r="AF41" s="315" t="s">
+      <c r="AF41" s="313" t="s">
         <v>62</v>
       </c>
       <c r="AG41" s="117" t="s">
@@ -6263,7 +6263,7 @@
       <c r="O42" s="138">
         <v>2605108147</v>
       </c>
-      <c r="P42" s="315">
+      <c r="P42" s="313">
         <v>2605109858</v>
       </c>
       <c r="Q42" s="139" t="s">
@@ -6285,10 +6285,10 @@
       <c r="AA42" s="6"/>
       <c r="AB42" s="6"/>
       <c r="AC42" s="24"/>
-      <c r="AD42" s="315"/>
-      <c r="AE42" s="315"/>
-      <c r="AF42" s="315"/>
-      <c r="AG42" s="316"/>
+      <c r="AD42" s="313"/>
+      <c r="AE42" s="313"/>
+      <c r="AF42" s="313"/>
+      <c r="AG42" s="314"/>
       <c r="AH42" s="80"/>
       <c r="AI42" s="80"/>
       <c r="AL42" s="25"/>
@@ -6331,7 +6331,7 @@
       <c r="O43" s="96">
         <v>2605109742</v>
       </c>
-      <c r="P43" s="315">
+      <c r="P43" s="313">
         <v>2605110213</v>
       </c>
       <c r="Q43" s="101" t="s">
@@ -6353,10 +6353,10 @@
       <c r="AA43" s="6"/>
       <c r="AB43" s="6"/>
       <c r="AC43" s="24"/>
-      <c r="AD43" s="315"/>
-      <c r="AE43" s="315"/>
-      <c r="AF43" s="315"/>
-      <c r="AG43" s="316"/>
+      <c r="AD43" s="313"/>
+      <c r="AE43" s="313"/>
+      <c r="AF43" s="313"/>
+      <c r="AG43" s="314"/>
       <c r="AH43" s="80"/>
       <c r="AI43" s="80"/>
       <c r="AL43" s="25"/>
@@ -6381,10 +6381,10 @@
       <c r="G44" s="7" t="s">
         <v>268</v>
       </c>
-      <c r="H44" s="315" t="s">
+      <c r="H44" s="313" t="s">
         <v>269</v>
       </c>
-      <c r="I44" s="317" t="s">
+      <c r="I44" s="315" t="s">
         <v>270</v>
       </c>
       <c r="J44" s="31"/>
@@ -6399,7 +6399,7 @@
       <c r="O44" s="96">
         <v>2605108514</v>
       </c>
-      <c r="P44" s="315">
+      <c r="P44" s="313">
         <v>2605109851</v>
       </c>
       <c r="Q44" s="100" t="s">
@@ -6422,9 +6422,9 @@
       <c r="AB44" s="6"/>
       <c r="AC44" s="24"/>
       <c r="AD44" s="39"/>
-      <c r="AE44" s="315"/>
-      <c r="AF44" s="315"/>
-      <c r="AG44" s="316"/>
+      <c r="AE44" s="313"/>
+      <c r="AF44" s="313"/>
+      <c r="AG44" s="314"/>
       <c r="AH44" s="80"/>
       <c r="AI44" s="80"/>
       <c r="AL44" s="25"/>
@@ -6449,10 +6449,10 @@
       <c r="G45" s="7" t="s">
         <v>272</v>
       </c>
-      <c r="H45" s="315" t="s">
+      <c r="H45" s="313" t="s">
         <v>273</v>
       </c>
-      <c r="I45" s="317" t="s">
+      <c r="I45" s="315" t="s">
         <v>274</v>
       </c>
       <c r="J45" s="31"/>
@@ -6467,7 +6467,7 @@
       <c r="O45" s="67">
         <v>2605109732</v>
       </c>
-      <c r="P45" s="315">
+      <c r="P45" s="313">
         <v>2605110161</v>
       </c>
       <c r="Q45" s="64" t="s">
@@ -6497,10 +6497,10 @@
       <c r="AE45" s="118">
         <v>46087.775949074072</v>
       </c>
-      <c r="AF45" s="315" t="s">
+      <c r="AF45" s="313" t="s">
         <v>62</v>
       </c>
-      <c r="AG45" s="316" t="s">
+      <c r="AG45" s="314" t="s">
         <v>63</v>
       </c>
       <c r="AH45" s="80"/>
@@ -6527,10 +6527,10 @@
       <c r="G46" s="7" t="s">
         <v>277</v>
       </c>
-      <c r="H46" s="315" t="s">
+      <c r="H46" s="313" t="s">
         <v>278</v>
       </c>
-      <c r="I46" s="317" t="s">
+      <c r="I46" s="315" t="s">
         <v>279</v>
       </c>
       <c r="J46" s="31"/>
@@ -6545,7 +6545,7 @@
       <c r="O46" s="67">
         <v>2605113276</v>
       </c>
-      <c r="P46" s="315">
+      <c r="P46" s="313">
         <v>2605114534</v>
       </c>
       <c r="Q46" s="100" t="s">
@@ -6567,10 +6567,10 @@
       <c r="AA46" s="6"/>
       <c r="AB46" s="6"/>
       <c r="AC46" s="24"/>
-      <c r="AD46" s="315"/>
-      <c r="AE46" s="315"/>
-      <c r="AF46" s="315"/>
-      <c r="AG46" s="316"/>
+      <c r="AD46" s="313"/>
+      <c r="AE46" s="313"/>
+      <c r="AF46" s="313"/>
+      <c r="AG46" s="314"/>
       <c r="AH46" s="80"/>
       <c r="AI46" s="80"/>
       <c r="AL46" s="25"/>
@@ -6613,7 +6613,7 @@
       <c r="O47" s="67">
         <v>2605113362</v>
       </c>
-      <c r="P47" s="315">
+      <c r="P47" s="313">
         <v>2605114515</v>
       </c>
       <c r="Q47" s="100" t="s">
@@ -6637,7 +6637,7 @@
       <c r="AC47" s="24"/>
       <c r="AD47" s="39"/>
       <c r="AE47" s="39"/>
-      <c r="AF47" s="315"/>
+      <c r="AF47" s="313"/>
       <c r="AG47" s="98"/>
       <c r="AH47" s="80"/>
       <c r="AI47" s="80"/>
@@ -6681,7 +6681,7 @@
       <c r="O48" s="67">
         <v>2605108328</v>
       </c>
-      <c r="P48" s="315">
+      <c r="P48" s="313">
         <v>2605109841</v>
       </c>
       <c r="Q48" s="102" t="s">
@@ -6711,7 +6711,7 @@
       <c r="AE48" s="118">
         <v>46087.596365740741</v>
       </c>
-      <c r="AF48" s="315" t="s">
+      <c r="AF48" s="313" t="s">
         <v>62</v>
       </c>
       <c r="AG48" s="117" t="s">
@@ -6759,7 +6759,7 @@
       <c r="O49" s="67">
         <v>2605109779</v>
       </c>
-      <c r="P49" s="315">
+      <c r="P49" s="313">
         <v>2605112451</v>
       </c>
       <c r="Q49" s="100" t="s">
@@ -6784,7 +6784,7 @@
       <c r="AD49" s="39"/>
       <c r="AE49" s="39"/>
       <c r="AF49" s="39"/>
-      <c r="AG49" s="316"/>
+      <c r="AG49" s="314"/>
       <c r="AH49" s="80"/>
       <c r="AI49" s="80"/>
       <c r="AL49" s="25"/>
@@ -6827,7 +6827,7 @@
       <c r="O50" s="67">
         <v>2605108680</v>
       </c>
-      <c r="P50" s="315">
+      <c r="P50" s="313">
         <v>2605110346</v>
       </c>
       <c r="Q50" s="139" t="s">
@@ -6860,7 +6860,7 @@
       <c r="AF50" s="120">
         <v>46086.831087962964</v>
       </c>
-      <c r="AG50" s="316" t="s">
+      <c r="AG50" s="314" t="s">
         <v>82</v>
       </c>
       <c r="AH50" s="80"/>
@@ -6905,7 +6905,7 @@
       <c r="O51" s="97">
         <v>2605113395</v>
       </c>
-      <c r="P51" s="315"/>
+      <c r="P51" s="313"/>
       <c r="Q51" s="143" t="s">
         <v>307</v>
       </c>
@@ -6928,10 +6928,10 @@
       <c r="AD51" s="39" t="s">
         <v>72</v>
       </c>
-      <c r="AE51" s="315" t="s">
+      <c r="AE51" s="313" t="s">
         <v>62</v>
       </c>
-      <c r="AF51" s="315" t="s">
+      <c r="AF51" s="313" t="s">
         <v>62</v>
       </c>
       <c r="AG51" s="98" t="s">
@@ -6979,7 +6979,7 @@
       <c r="O52" s="97">
         <v>2605110890</v>
       </c>
-      <c r="P52" s="315">
+      <c r="P52" s="313">
         <v>2605112505</v>
       </c>
       <c r="Q52" s="100" t="s">
@@ -7006,10 +7006,10 @@
       <c r="AD52" s="52">
         <v>46085.809814814813</v>
       </c>
-      <c r="AE52" s="318">
+      <c r="AE52" s="316">
         <v>46087.775717592594</v>
       </c>
-      <c r="AF52" s="315" t="s">
+      <c r="AF52" s="313" t="s">
         <v>62</v>
       </c>
       <c r="AG52" s="117" t="s">
@@ -7057,7 +7057,7 @@
       <c r="O53" s="113">
         <v>2605113776</v>
       </c>
-      <c r="P53" s="315">
+      <c r="P53" s="313">
         <v>2605114358</v>
       </c>
       <c r="Q53" s="112" t="s">
@@ -7080,9 +7080,9 @@
       <c r="AB53" s="6"/>
       <c r="AC53" s="24"/>
       <c r="AD53" s="116"/>
-      <c r="AE53" s="315"/>
-      <c r="AF53" s="315"/>
-      <c r="AG53" s="316"/>
+      <c r="AE53" s="313"/>
+      <c r="AF53" s="313"/>
+      <c r="AG53" s="314"/>
       <c r="AH53" s="80"/>
       <c r="AI53" s="80"/>
       <c r="AL53" s="25"/>
@@ -7125,7 +7125,7 @@
       <c r="O54" s="113">
         <v>2605113989</v>
       </c>
-      <c r="P54" s="315">
+      <c r="P54" s="313">
         <v>2605114359</v>
       </c>
       <c r="Q54" s="100" t="s">
@@ -7147,10 +7147,10 @@
       <c r="AA54" s="26"/>
       <c r="AB54" s="26"/>
       <c r="AC54" s="37"/>
-      <c r="AD54" s="315"/>
-      <c r="AE54" s="315"/>
-      <c r="AF54" s="315"/>
-      <c r="AG54" s="316"/>
+      <c r="AD54" s="313"/>
+      <c r="AE54" s="313"/>
+      <c r="AF54" s="313"/>
+      <c r="AG54" s="314"/>
       <c r="AH54" s="80"/>
       <c r="AI54" s="80"/>
       <c r="AL54" s="38"/>
@@ -7189,7 +7189,7 @@
         <v>72</v>
       </c>
       <c r="O55" s="136"/>
-      <c r="P55" s="315"/>
+      <c r="P55" s="313"/>
       <c r="Q55" s="104"/>
       <c r="R55" s="42"/>
       <c r="S55" s="86" t="s">
@@ -7253,7 +7253,7 @@
       <c r="O56" s="64">
         <v>2605111955</v>
       </c>
-      <c r="P56" s="315">
+      <c r="P56" s="313">
         <v>2605112639</v>
       </c>
       <c r="Q56" s="103" t="s">
@@ -7303,7 +7303,7 @@
       <c r="G57" s="6" t="s">
         <v>335</v>
       </c>
-      <c r="H57" s="315" t="s">
+      <c r="H57" s="313" t="s">
         <v>336</v>
       </c>
       <c r="I57" s="6" t="s">
@@ -7321,7 +7321,7 @@
       <c r="O57" s="67">
         <v>2605111677</v>
       </c>
-      <c r="P57" s="315">
+      <c r="P57" s="313">
         <v>2605112425</v>
       </c>
       <c r="Q57" s="100" t="s">
@@ -7343,10 +7343,10 @@
       <c r="AA57" s="6"/>
       <c r="AB57" s="6"/>
       <c r="AC57" s="6"/>
-      <c r="AD57" s="317"/>
-      <c r="AE57" s="317"/>
-      <c r="AF57" s="317"/>
-      <c r="AG57" s="319"/>
+      <c r="AD57" s="315"/>
+      <c r="AE57" s="315"/>
+      <c r="AF57" s="315"/>
+      <c r="AG57" s="317"/>
       <c r="AL57" s="25"/>
       <c r="AM57" s="91"/>
     </row>
@@ -7369,10 +7369,10 @@
       <c r="G58" s="6" t="s">
         <v>340</v>
       </c>
-      <c r="H58" s="315" t="s">
+      <c r="H58" s="313" t="s">
         <v>341</v>
       </c>
-      <c r="I58" s="317" t="s">
+      <c r="I58" s="315" t="s">
         <v>342</v>
       </c>
       <c r="J58" s="31"/>
@@ -7387,7 +7387,7 @@
       <c r="O58" s="67">
         <v>2605113022</v>
       </c>
-      <c r="P58" s="315">
+      <c r="P58" s="313">
         <v>2605114351</v>
       </c>
       <c r="Q58" s="112" t="s">
@@ -7409,10 +7409,10 @@
       <c r="AA58" s="6"/>
       <c r="AB58" s="6"/>
       <c r="AC58" s="6"/>
-      <c r="AD58" s="317"/>
-      <c r="AE58" s="317"/>
-      <c r="AF58" s="317"/>
-      <c r="AG58" s="319"/>
+      <c r="AD58" s="315"/>
+      <c r="AE58" s="315"/>
+      <c r="AF58" s="315"/>
+      <c r="AG58" s="317"/>
       <c r="AL58" s="25"/>
       <c r="AM58" s="91"/>
     </row>
@@ -7435,8 +7435,8 @@
       <c r="G59" s="233" t="s">
         <v>345</v>
       </c>
-      <c r="H59" s="315"/>
-      <c r="I59" s="317"/>
+      <c r="H59" s="313"/>
+      <c r="I59" s="315"/>
       <c r="J59" s="31"/>
       <c r="K59" s="6"/>
       <c r="L59" s="6" t="s">
@@ -7449,7 +7449,7 @@
       <c r="O59" s="61">
         <v>2605114146</v>
       </c>
-      <c r="P59" s="315"/>
+      <c r="P59" s="313"/>
       <c r="Q59" s="104"/>
       <c r="R59" s="24"/>
       <c r="S59" s="11" t="s">
@@ -7458,7 +7458,7 @@
       <c r="T59" s="50">
         <v>4090180261</v>
       </c>
-      <c r="U59" s="317"/>
+      <c r="U59" s="315"/>
       <c r="V59" s="31"/>
       <c r="W59" s="6"/>
       <c r="X59" s="6"/>
@@ -7467,10 +7467,10 @@
       <c r="AA59" s="6"/>
       <c r="AB59" s="6"/>
       <c r="AC59" s="6"/>
-      <c r="AD59" s="317"/>
-      <c r="AE59" s="317"/>
-      <c r="AF59" s="317"/>
-      <c r="AG59" s="319"/>
+      <c r="AD59" s="315"/>
+      <c r="AE59" s="315"/>
+      <c r="AF59" s="315"/>
+      <c r="AG59" s="317"/>
       <c r="AL59" s="25"/>
       <c r="AM59" s="91"/>
     </row>
@@ -7490,13 +7490,13 @@
       <c r="F60" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="G60" s="317" t="s">
+      <c r="G60" s="315" t="s">
         <v>347</v>
       </c>
-      <c r="H60" s="315" t="s">
+      <c r="H60" s="313" t="s">
         <v>348</v>
       </c>
-      <c r="I60" s="317" t="s">
+      <c r="I60" s="315" t="s">
         <v>349</v>
       </c>
       <c r="J60" s="31"/>
@@ -7524,7 +7524,7 @@
       <c r="T60" s="244">
         <v>4090180263</v>
       </c>
-      <c r="U60" s="317"/>
+      <c r="U60" s="315"/>
       <c r="V60" s="31"/>
       <c r="W60" s="6"/>
       <c r="X60" s="6"/>
@@ -7533,10 +7533,10 @@
       <c r="AA60" s="6"/>
       <c r="AB60" s="6"/>
       <c r="AC60" s="6"/>
-      <c r="AD60" s="317"/>
-      <c r="AE60" s="317"/>
-      <c r="AF60" s="317"/>
-      <c r="AG60" s="319"/>
+      <c r="AD60" s="315"/>
+      <c r="AE60" s="315"/>
+      <c r="AF60" s="315"/>
+      <c r="AG60" s="317"/>
       <c r="AL60" s="25"/>
       <c r="AM60" s="91"/>
     </row>
@@ -7556,11 +7556,11 @@
       <c r="F61" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="G61" s="317" t="s">
+      <c r="G61" s="315" t="s">
         <v>352</v>
       </c>
-      <c r="H61" s="315"/>
-      <c r="I61" s="317"/>
+      <c r="H61" s="313"/>
+      <c r="I61" s="315"/>
       <c r="J61" s="31"/>
       <c r="K61" s="6"/>
       <c r="L61" s="6" t="s">
@@ -7579,7 +7579,7 @@
       <c r="T61" s="50">
         <v>4090180265</v>
       </c>
-      <c r="U61" s="317"/>
+      <c r="U61" s="315"/>
       <c r="V61" s="31"/>
       <c r="W61" s="6"/>
       <c r="X61" s="6"/>
@@ -7588,10 +7588,10 @@
       <c r="AA61" s="6"/>
       <c r="AB61" s="6"/>
       <c r="AC61" s="6"/>
-      <c r="AD61" s="317"/>
-      <c r="AE61" s="317"/>
-      <c r="AF61" s="317"/>
-      <c r="AG61" s="319"/>
+      <c r="AD61" s="315"/>
+      <c r="AE61" s="315"/>
+      <c r="AF61" s="315"/>
+      <c r="AG61" s="317"/>
       <c r="AL61" s="25"/>
       <c r="AM61" s="91"/>
     </row>
@@ -7611,11 +7611,11 @@
       <c r="F62" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="G62" s="317" t="s">
+      <c r="G62" s="315" t="s">
         <v>355</v>
       </c>
-      <c r="H62" s="315"/>
-      <c r="I62" s="317"/>
+      <c r="H62" s="313"/>
+      <c r="I62" s="315"/>
       <c r="J62" s="31"/>
       <c r="K62" s="6"/>
       <c r="L62" s="6"/>
@@ -7632,7 +7632,7 @@
       <c r="T62" s="50">
         <v>4090180284</v>
       </c>
-      <c r="U62" s="317"/>
+      <c r="U62" s="315"/>
       <c r="V62" s="31"/>
       <c r="W62" s="6"/>
       <c r="X62" s="6"/>
@@ -7641,10 +7641,10 @@
       <c r="AA62" s="6"/>
       <c r="AB62" s="6"/>
       <c r="AC62" s="6"/>
-      <c r="AD62" s="317"/>
-      <c r="AE62" s="317"/>
-      <c r="AF62" s="317"/>
-      <c r="AG62" s="319"/>
+      <c r="AD62" s="315"/>
+      <c r="AE62" s="315"/>
+      <c r="AF62" s="315"/>
+      <c r="AG62" s="317"/>
       <c r="AL62" s="25"/>
       <c r="AM62" s="91"/>
     </row>
@@ -7664,11 +7664,11 @@
       <c r="F63" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="G63" s="317" t="s">
+      <c r="G63" s="315" t="s">
         <v>357</v>
       </c>
-      <c r="H63" s="315"/>
-      <c r="I63" s="317"/>
+      <c r="H63" s="313"/>
+      <c r="I63" s="315"/>
       <c r="J63" s="31"/>
       <c r="K63" s="6"/>
       <c r="L63" s="6"/>
@@ -7685,7 +7685,7 @@
       <c r="T63" s="50">
         <v>4090180286</v>
       </c>
-      <c r="U63" s="317"/>
+      <c r="U63" s="315"/>
       <c r="V63" s="31"/>
       <c r="W63" s="6"/>
       <c r="X63" s="6"/>
@@ -7694,10 +7694,10 @@
       <c r="AA63" s="6"/>
       <c r="AB63" s="6"/>
       <c r="AC63" s="6"/>
-      <c r="AD63" s="317"/>
-      <c r="AE63" s="317"/>
-      <c r="AF63" s="317"/>
-      <c r="AG63" s="319"/>
+      <c r="AD63" s="315"/>
+      <c r="AE63" s="315"/>
+      <c r="AF63" s="315"/>
+      <c r="AG63" s="317"/>
       <c r="AL63" s="25"/>
       <c r="AM63" s="91"/>
     </row>
@@ -7711,9 +7711,9 @@
       <c r="D64" s="6"/>
       <c r="E64" s="6"/>
       <c r="F64" s="6"/>
-      <c r="G64" s="317"/>
-      <c r="H64" s="315"/>
-      <c r="I64" s="317"/>
+      <c r="G64" s="315"/>
+      <c r="H64" s="313"/>
+      <c r="I64" s="315"/>
       <c r="J64" s="31"/>
       <c r="K64" s="6"/>
       <c r="L64" s="6"/>
@@ -7724,7 +7724,7 @@
       <c r="R64" s="6"/>
       <c r="S64" s="140"/>
       <c r="T64" s="245"/>
-      <c r="U64" s="320"/>
+      <c r="U64" s="318"/>
       <c r="V64" s="6"/>
       <c r="W64" s="6"/>
       <c r="X64" s="6"/>
@@ -7733,10 +7733,10 @@
       <c r="AA64" s="6"/>
       <c r="AB64" s="6"/>
       <c r="AC64" s="6"/>
-      <c r="AD64" s="317"/>
-      <c r="AE64" s="317"/>
-      <c r="AF64" s="317"/>
-      <c r="AG64" s="319"/>
+      <c r="AD64" s="315"/>
+      <c r="AE64" s="315"/>
+      <c r="AF64" s="315"/>
+      <c r="AG64" s="317"/>
       <c r="AL64" s="25"/>
       <c r="AM64" s="91"/>
     </row>
@@ -7750,9 +7750,9 @@
       <c r="D65" s="6"/>
       <c r="E65" s="6"/>
       <c r="F65" s="6"/>
-      <c r="G65" s="317"/>
-      <c r="H65" s="315"/>
-      <c r="I65" s="317"/>
+      <c r="G65" s="315"/>
+      <c r="H65" s="313"/>
+      <c r="I65" s="315"/>
       <c r="J65" s="31"/>
       <c r="K65" s="6"/>
       <c r="L65" s="6"/>
@@ -7763,7 +7763,7 @@
       <c r="R65" s="6"/>
       <c r="S65" s="6"/>
       <c r="T65" s="50"/>
-      <c r="U65" s="317"/>
+      <c r="U65" s="315"/>
       <c r="V65" s="6"/>
       <c r="W65" s="6"/>
       <c r="X65" s="6"/>
@@ -7772,10 +7772,10 @@
       <c r="AA65" s="6"/>
       <c r="AB65" s="6"/>
       <c r="AC65" s="6"/>
-      <c r="AD65" s="317"/>
-      <c r="AE65" s="317"/>
-      <c r="AF65" s="317"/>
-      <c r="AG65" s="319"/>
+      <c r="AD65" s="315"/>
+      <c r="AE65" s="315"/>
+      <c r="AF65" s="315"/>
+      <c r="AG65" s="317"/>
       <c r="AL65" s="25"/>
       <c r="AM65" s="91"/>
     </row>
@@ -7789,9 +7789,9 @@
       <c r="D66" s="6"/>
       <c r="E66" s="6"/>
       <c r="F66" s="6"/>
-      <c r="G66" s="317"/>
-      <c r="H66" s="315"/>
-      <c r="I66" s="317"/>
+      <c r="G66" s="315"/>
+      <c r="H66" s="313"/>
+      <c r="I66" s="315"/>
       <c r="J66" s="31"/>
       <c r="K66" s="6"/>
       <c r="L66" s="6"/>
@@ -7802,7 +7802,7 @@
       <c r="R66" s="6"/>
       <c r="S66" s="6"/>
       <c r="T66" s="50"/>
-      <c r="U66" s="317"/>
+      <c r="U66" s="315"/>
       <c r="V66" s="6"/>
       <c r="W66" s="6"/>
       <c r="X66" s="6"/>
@@ -7811,10 +7811,10 @@
       <c r="AA66" s="6"/>
       <c r="AB66" s="6"/>
       <c r="AC66" s="6"/>
-      <c r="AD66" s="317"/>
-      <c r="AE66" s="317"/>
-      <c r="AF66" s="317"/>
-      <c r="AG66" s="319"/>
+      <c r="AD66" s="315"/>
+      <c r="AE66" s="315"/>
+      <c r="AF66" s="315"/>
+      <c r="AG66" s="317"/>
       <c r="AL66" s="25"/>
       <c r="AM66" s="91"/>
     </row>
@@ -7828,9 +7828,9 @@
       <c r="D67" s="6"/>
       <c r="E67" s="6"/>
       <c r="F67" s="6"/>
-      <c r="G67" s="317"/>
-      <c r="H67" s="315"/>
-      <c r="I67" s="317"/>
+      <c r="G67" s="315"/>
+      <c r="H67" s="313"/>
+      <c r="I67" s="315"/>
       <c r="J67" s="31"/>
       <c r="K67" s="6"/>
       <c r="L67" s="6"/>
@@ -7841,7 +7841,7 @@
       <c r="R67" s="6"/>
       <c r="S67" s="6"/>
       <c r="T67" s="50"/>
-      <c r="U67" s="317"/>
+      <c r="U67" s="315"/>
       <c r="V67" s="6"/>
       <c r="W67" s="6"/>
       <c r="X67" s="6"/>
@@ -7850,10 +7850,10 @@
       <c r="AA67" s="6"/>
       <c r="AB67" s="6"/>
       <c r="AC67" s="6"/>
-      <c r="AD67" s="317"/>
-      <c r="AE67" s="317"/>
-      <c r="AF67" s="317"/>
-      <c r="AG67" s="319"/>
+      <c r="AD67" s="315"/>
+      <c r="AE67" s="315"/>
+      <c r="AF67" s="315"/>
+      <c r="AG67" s="317"/>
       <c r="AL67" s="25"/>
       <c r="AM67" s="91"/>
     </row>
@@ -7863,9 +7863,9 @@
       <c r="D68" s="6"/>
       <c r="E68" s="6"/>
       <c r="F68" s="6"/>
-      <c r="G68" s="317"/>
-      <c r="H68" s="315"/>
-      <c r="I68" s="317"/>
+      <c r="G68" s="315"/>
+      <c r="H68" s="313"/>
+      <c r="I68" s="315"/>
       <c r="J68" s="31"/>
       <c r="K68" s="6"/>
       <c r="L68" s="6"/>
@@ -7876,7 +7876,7 @@
       <c r="R68" s="6"/>
       <c r="S68" s="6"/>
       <c r="T68" s="50"/>
-      <c r="U68" s="317"/>
+      <c r="U68" s="315"/>
       <c r="V68" s="6"/>
       <c r="W68" s="6"/>
       <c r="X68" s="6"/>
@@ -7885,10 +7885,10 @@
       <c r="AA68" s="6"/>
       <c r="AB68" s="6"/>
       <c r="AC68" s="6"/>
-      <c r="AD68" s="317"/>
-      <c r="AE68" s="317"/>
-      <c r="AF68" s="317"/>
-      <c r="AG68" s="319"/>
+      <c r="AD68" s="315"/>
+      <c r="AE68" s="315"/>
+      <c r="AF68" s="315"/>
+      <c r="AG68" s="317"/>
       <c r="AL68" s="25"/>
       <c r="AM68" s="91"/>
     </row>
@@ -7898,9 +7898,9 @@
       <c r="D69" s="6"/>
       <c r="E69" s="6"/>
       <c r="F69" s="6"/>
-      <c r="G69" s="317"/>
-      <c r="H69" s="315"/>
-      <c r="I69" s="317"/>
+      <c r="G69" s="315"/>
+      <c r="H69" s="313"/>
+      <c r="I69" s="315"/>
       <c r="J69" s="31"/>
       <c r="K69" s="6"/>
       <c r="L69" s="6"/>
@@ -7911,7 +7911,7 @@
       <c r="R69" s="6"/>
       <c r="S69" s="6"/>
       <c r="T69" s="50"/>
-      <c r="U69" s="317"/>
+      <c r="U69" s="315"/>
       <c r="V69" s="6"/>
       <c r="W69" s="6"/>
       <c r="X69" s="6"/>
@@ -7920,10 +7920,10 @@
       <c r="AA69" s="6"/>
       <c r="AB69" s="6"/>
       <c r="AC69" s="6"/>
-      <c r="AD69" s="317"/>
-      <c r="AE69" s="317"/>
-      <c r="AF69" s="317"/>
-      <c r="AG69" s="319"/>
+      <c r="AD69" s="315"/>
+      <c r="AE69" s="315"/>
+      <c r="AF69" s="315"/>
+      <c r="AG69" s="317"/>
       <c r="AL69" s="25"/>
       <c r="AM69" s="91"/>
     </row>
@@ -7933,9 +7933,9 @@
       <c r="D70" s="6"/>
       <c r="E70" s="6"/>
       <c r="F70" s="6"/>
-      <c r="G70" s="317"/>
-      <c r="H70" s="315"/>
-      <c r="I70" s="317"/>
+      <c r="G70" s="315"/>
+      <c r="H70" s="313"/>
+      <c r="I70" s="315"/>
       <c r="J70" s="31"/>
       <c r="K70" s="6"/>
       <c r="L70" s="6"/>
@@ -7946,7 +7946,7 @@
       <c r="R70" s="6"/>
       <c r="S70" s="6"/>
       <c r="T70" s="50"/>
-      <c r="U70" s="317"/>
+      <c r="U70" s="315"/>
       <c r="V70" s="6"/>
       <c r="W70" s="6"/>
       <c r="X70" s="6"/>
@@ -7955,10 +7955,10 @@
       <c r="AA70" s="6"/>
       <c r="AB70" s="6"/>
       <c r="AC70" s="6"/>
-      <c r="AD70" s="317"/>
-      <c r="AE70" s="317"/>
-      <c r="AF70" s="317"/>
-      <c r="AG70" s="319"/>
+      <c r="AD70" s="315"/>
+      <c r="AE70" s="315"/>
+      <c r="AF70" s="315"/>
+      <c r="AG70" s="317"/>
       <c r="AL70" s="25"/>
       <c r="AM70" s="91"/>
     </row>
@@ -7968,9 +7968,9 @@
       <c r="D71" s="6"/>
       <c r="E71" s="6"/>
       <c r="F71" s="6"/>
-      <c r="G71" s="317"/>
-      <c r="H71" s="315"/>
-      <c r="I71" s="317"/>
+      <c r="G71" s="315"/>
+      <c r="H71" s="313"/>
+      <c r="I71" s="315"/>
       <c r="J71" s="31"/>
       <c r="K71" s="6"/>
       <c r="L71" s="6"/>
@@ -7981,7 +7981,7 @@
       <c r="R71" s="6"/>
       <c r="S71" s="6"/>
       <c r="T71" s="50"/>
-      <c r="U71" s="317"/>
+      <c r="U71" s="315"/>
       <c r="V71" s="6"/>
       <c r="W71" s="6"/>
       <c r="X71" s="6"/>
@@ -7990,10 +7990,10 @@
       <c r="AA71" s="6"/>
       <c r="AB71" s="6"/>
       <c r="AC71" s="6"/>
-      <c r="AD71" s="317"/>
-      <c r="AE71" s="317"/>
-      <c r="AF71" s="317"/>
-      <c r="AG71" s="319"/>
+      <c r="AD71" s="315"/>
+      <c r="AE71" s="315"/>
+      <c r="AF71" s="315"/>
+      <c r="AG71" s="317"/>
       <c r="AL71" s="25"/>
       <c r="AM71" s="91"/>
     </row>
@@ -8003,9 +8003,9 @@
       <c r="D72" s="6"/>
       <c r="E72" s="6"/>
       <c r="F72" s="6"/>
-      <c r="G72" s="317"/>
-      <c r="H72" s="315"/>
-      <c r="I72" s="317"/>
+      <c r="G72" s="315"/>
+      <c r="H72" s="313"/>
+      <c r="I72" s="315"/>
       <c r="J72" s="31"/>
       <c r="K72" s="6"/>
       <c r="L72" s="6"/>
@@ -8016,7 +8016,7 @@
       <c r="R72" s="6"/>
       <c r="S72" s="6"/>
       <c r="T72" s="50"/>
-      <c r="U72" s="317"/>
+      <c r="U72" s="315"/>
       <c r="V72" s="6"/>
       <c r="W72" s="6"/>
       <c r="X72" s="6"/>
@@ -8025,10 +8025,10 @@
       <c r="AA72" s="6"/>
       <c r="AB72" s="6"/>
       <c r="AC72" s="6"/>
-      <c r="AD72" s="317"/>
-      <c r="AE72" s="317"/>
-      <c r="AF72" s="317"/>
-      <c r="AG72" s="319"/>
+      <c r="AD72" s="315"/>
+      <c r="AE72" s="315"/>
+      <c r="AF72" s="315"/>
+      <c r="AG72" s="317"/>
       <c r="AL72" s="25"/>
       <c r="AM72" s="91"/>
     </row>
@@ -8038,9 +8038,9 @@
       <c r="D73" s="6"/>
       <c r="E73" s="6"/>
       <c r="F73" s="6"/>
-      <c r="G73" s="317"/>
-      <c r="H73" s="315"/>
-      <c r="I73" s="317"/>
+      <c r="G73" s="315"/>
+      <c r="H73" s="313"/>
+      <c r="I73" s="315"/>
       <c r="J73" s="31"/>
       <c r="K73" s="6"/>
       <c r="L73" s="6"/>
@@ -8051,7 +8051,7 @@
       <c r="R73" s="6"/>
       <c r="S73" s="6"/>
       <c r="T73" s="50"/>
-      <c r="U73" s="317"/>
+      <c r="U73" s="315"/>
       <c r="V73" s="6"/>
       <c r="W73" s="6"/>
       <c r="X73" s="6"/>
@@ -8060,10 +8060,10 @@
       <c r="AA73" s="6"/>
       <c r="AB73" s="6"/>
       <c r="AC73" s="6"/>
-      <c r="AD73" s="317"/>
-      <c r="AE73" s="317"/>
-      <c r="AF73" s="317"/>
-      <c r="AG73" s="319"/>
+      <c r="AD73" s="315"/>
+      <c r="AE73" s="315"/>
+      <c r="AF73" s="315"/>
+      <c r="AG73" s="317"/>
       <c r="AL73" s="25"/>
       <c r="AM73" s="91"/>
     </row>
@@ -8073,9 +8073,9 @@
       <c r="D74" s="6"/>
       <c r="E74" s="6"/>
       <c r="F74" s="6"/>
-      <c r="G74" s="317"/>
-      <c r="H74" s="315"/>
-      <c r="I74" s="317"/>
+      <c r="G74" s="315"/>
+      <c r="H74" s="313"/>
+      <c r="I74" s="315"/>
       <c r="J74" s="31"/>
       <c r="K74" s="6"/>
       <c r="L74" s="6"/>
@@ -8086,7 +8086,7 @@
       <c r="R74" s="6"/>
       <c r="S74" s="6"/>
       <c r="T74" s="50"/>
-      <c r="U74" s="317"/>
+      <c r="U74" s="315"/>
       <c r="V74" s="6"/>
       <c r="W74" s="6"/>
       <c r="X74" s="6"/>
@@ -8095,10 +8095,10 @@
       <c r="AA74" s="6"/>
       <c r="AB74" s="6"/>
       <c r="AC74" s="6"/>
-      <c r="AD74" s="317"/>
-      <c r="AE74" s="317"/>
-      <c r="AF74" s="317"/>
-      <c r="AG74" s="319"/>
+      <c r="AD74" s="315"/>
+      <c r="AE74" s="315"/>
+      <c r="AF74" s="315"/>
+      <c r="AG74" s="317"/>
       <c r="AL74" s="25"/>
       <c r="AM74" s="91"/>
     </row>
@@ -8108,9 +8108,9 @@
       <c r="D75" s="6"/>
       <c r="E75" s="6"/>
       <c r="F75" s="6"/>
-      <c r="G75" s="317"/>
-      <c r="H75" s="315"/>
-      <c r="I75" s="317"/>
+      <c r="G75" s="315"/>
+      <c r="H75" s="313"/>
+      <c r="I75" s="315"/>
       <c r="J75" s="31"/>
       <c r="K75" s="6"/>
       <c r="L75" s="6"/>
@@ -8121,7 +8121,7 @@
       <c r="R75" s="6"/>
       <c r="S75" s="6"/>
       <c r="T75" s="50"/>
-      <c r="U75" s="317"/>
+      <c r="U75" s="315"/>
       <c r="V75" s="6"/>
       <c r="W75" s="6"/>
       <c r="X75" s="6"/>
@@ -8130,10 +8130,10 @@
       <c r="AA75" s="6"/>
       <c r="AB75" s="6"/>
       <c r="AC75" s="6"/>
-      <c r="AD75" s="317"/>
-      <c r="AE75" s="317"/>
-      <c r="AF75" s="317"/>
-      <c r="AG75" s="319"/>
+      <c r="AD75" s="315"/>
+      <c r="AE75" s="315"/>
+      <c r="AF75" s="315"/>
+      <c r="AG75" s="317"/>
       <c r="AL75" s="25"/>
       <c r="AM75" s="91"/>
     </row>
@@ -8143,9 +8143,9 @@
       <c r="D76" s="6"/>
       <c r="E76" s="6"/>
       <c r="F76" s="6"/>
-      <c r="G76" s="317"/>
-      <c r="H76" s="315"/>
-      <c r="I76" s="317"/>
+      <c r="G76" s="315"/>
+      <c r="H76" s="313"/>
+      <c r="I76" s="315"/>
       <c r="J76" s="31"/>
       <c r="K76" s="6"/>
       <c r="L76" s="6"/>
@@ -8155,8 +8155,8 @@
       <c r="Q76" s="104"/>
       <c r="R76" s="6"/>
       <c r="S76" s="6"/>
-      <c r="T76" s="317"/>
-      <c r="U76" s="317"/>
+      <c r="T76" s="315"/>
+      <c r="U76" s="315"/>
       <c r="V76" s="6"/>
       <c r="W76" s="6"/>
       <c r="X76" s="6"/>
@@ -8165,10 +8165,10 @@
       <c r="AA76" s="6"/>
       <c r="AB76" s="6"/>
       <c r="AC76" s="6"/>
-      <c r="AD76" s="317"/>
-      <c r="AE76" s="317"/>
-      <c r="AF76" s="317"/>
-      <c r="AG76" s="319"/>
+      <c r="AD76" s="315"/>
+      <c r="AE76" s="315"/>
+      <c r="AF76" s="315"/>
+      <c r="AG76" s="317"/>
       <c r="AL76" s="25"/>
       <c r="AM76" s="91"/>
     </row>
@@ -8178,9 +8178,9 @@
       <c r="D77" s="6"/>
       <c r="E77" s="6"/>
       <c r="F77" s="6"/>
-      <c r="G77" s="317"/>
-      <c r="H77" s="315"/>
-      <c r="I77" s="317"/>
+      <c r="G77" s="315"/>
+      <c r="H77" s="313"/>
+      <c r="I77" s="315"/>
       <c r="J77" s="31"/>
       <c r="K77" s="6"/>
       <c r="L77" s="6"/>
@@ -8190,8 +8190,8 @@
       <c r="Q77" s="104"/>
       <c r="R77" s="6"/>
       <c r="S77" s="6"/>
-      <c r="T77" s="317"/>
-      <c r="U77" s="317"/>
+      <c r="T77" s="315"/>
+      <c r="U77" s="315"/>
       <c r="V77" s="6"/>
       <c r="W77" s="6"/>
       <c r="X77" s="6"/>
@@ -8200,10 +8200,10 @@
       <c r="AA77" s="6"/>
       <c r="AB77" s="6"/>
       <c r="AC77" s="6"/>
-      <c r="AD77" s="317"/>
-      <c r="AE77" s="317"/>
-      <c r="AF77" s="317"/>
-      <c r="AG77" s="319"/>
+      <c r="AD77" s="315"/>
+      <c r="AE77" s="315"/>
+      <c r="AF77" s="315"/>
+      <c r="AG77" s="317"/>
       <c r="AL77" s="25"/>
       <c r="AM77" s="91"/>
     </row>
@@ -8213,9 +8213,9 @@
       <c r="D78" s="6"/>
       <c r="E78" s="6"/>
       <c r="F78" s="6"/>
-      <c r="G78" s="317"/>
-      <c r="H78" s="315"/>
-      <c r="I78" s="317"/>
+      <c r="G78" s="315"/>
+      <c r="H78" s="313"/>
+      <c r="I78" s="315"/>
       <c r="J78" s="31"/>
       <c r="K78" s="6"/>
       <c r="L78" s="6"/>
@@ -8225,7 +8225,7 @@
       <c r="Q78" s="104"/>
       <c r="R78" s="6"/>
       <c r="S78" s="6"/>
-      <c r="T78" s="317"/>
+      <c r="T78" s="315"/>
       <c r="U78" s="6"/>
       <c r="V78" s="6"/>
       <c r="W78" s="6"/>
@@ -8235,10 +8235,10 @@
       <c r="AA78" s="6"/>
       <c r="AB78" s="6"/>
       <c r="AC78" s="6"/>
-      <c r="AD78" s="317"/>
-      <c r="AE78" s="317"/>
-      <c r="AF78" s="317"/>
-      <c r="AG78" s="319"/>
+      <c r="AD78" s="315"/>
+      <c r="AE78" s="315"/>
+      <c r="AF78" s="315"/>
+      <c r="AG78" s="317"/>
       <c r="AL78" s="25"/>
       <c r="AM78" s="91"/>
     </row>
@@ -8248,9 +8248,9 @@
       <c r="D79" s="6"/>
       <c r="E79" s="6"/>
       <c r="F79" s="6"/>
-      <c r="G79" s="317"/>
-      <c r="H79" s="315"/>
-      <c r="I79" s="317"/>
+      <c r="G79" s="315"/>
+      <c r="H79" s="313"/>
+      <c r="I79" s="315"/>
       <c r="J79" s="31"/>
       <c r="K79" s="6"/>
       <c r="L79" s="6"/>
@@ -8260,7 +8260,7 @@
       <c r="Q79" s="104"/>
       <c r="R79" s="6"/>
       <c r="S79" s="6"/>
-      <c r="T79" s="317"/>
+      <c r="T79" s="315"/>
       <c r="U79" s="6"/>
       <c r="V79" s="6"/>
       <c r="W79" s="6"/>
@@ -8270,10 +8270,10 @@
       <c r="AA79" s="6"/>
       <c r="AB79" s="6"/>
       <c r="AC79" s="6"/>
-      <c r="AD79" s="317"/>
-      <c r="AE79" s="317"/>
-      <c r="AF79" s="317"/>
-      <c r="AG79" s="319"/>
+      <c r="AD79" s="315"/>
+      <c r="AE79" s="315"/>
+      <c r="AF79" s="315"/>
+      <c r="AG79" s="317"/>
       <c r="AL79" s="25"/>
       <c r="AM79" s="91"/>
     </row>
@@ -8283,9 +8283,9 @@
       <c r="D80" s="6"/>
       <c r="E80" s="6"/>
       <c r="F80" s="6"/>
-      <c r="G80" s="317"/>
-      <c r="H80" s="315"/>
-      <c r="I80" s="317"/>
+      <c r="G80" s="315"/>
+      <c r="H80" s="313"/>
+      <c r="I80" s="315"/>
       <c r="J80" s="31"/>
       <c r="K80" s="6"/>
       <c r="L80" s="6"/>
@@ -8295,7 +8295,7 @@
       <c r="Q80" s="104"/>
       <c r="R80" s="6"/>
       <c r="S80" s="6"/>
-      <c r="T80" s="317"/>
+      <c r="T80" s="315"/>
       <c r="U80" s="6"/>
       <c r="V80" s="6"/>
       <c r="W80" s="6"/>
@@ -8305,10 +8305,10 @@
       <c r="AA80" s="6"/>
       <c r="AB80" s="6"/>
       <c r="AC80" s="6"/>
-      <c r="AD80" s="317"/>
-      <c r="AE80" s="317"/>
-      <c r="AF80" s="317"/>
-      <c r="AG80" s="319"/>
+      <c r="AD80" s="315"/>
+      <c r="AE80" s="315"/>
+      <c r="AF80" s="315"/>
+      <c r="AG80" s="317"/>
       <c r="AL80" s="25"/>
       <c r="AM80" s="91"/>
     </row>
@@ -8318,9 +8318,9 @@
       <c r="D81" s="6"/>
       <c r="E81" s="6"/>
       <c r="F81" s="6"/>
-      <c r="G81" s="317"/>
-      <c r="H81" s="315"/>
-      <c r="I81" s="317"/>
+      <c r="G81" s="315"/>
+      <c r="H81" s="313"/>
+      <c r="I81" s="315"/>
       <c r="J81" s="31"/>
       <c r="K81" s="6"/>
       <c r="L81" s="6"/>
@@ -8330,7 +8330,7 @@
       <c r="Q81" s="104"/>
       <c r="R81" s="6"/>
       <c r="S81" s="6"/>
-      <c r="T81" s="317"/>
+      <c r="T81" s="315"/>
       <c r="U81" s="6"/>
       <c r="V81" s="6"/>
       <c r="W81" s="6"/>
@@ -8340,10 +8340,10 @@
       <c r="AA81" s="6"/>
       <c r="AB81" s="6"/>
       <c r="AC81" s="6"/>
-      <c r="AD81" s="317"/>
-      <c r="AE81" s="317"/>
-      <c r="AF81" s="317"/>
-      <c r="AG81" s="319"/>
+      <c r="AD81" s="315"/>
+      <c r="AE81" s="315"/>
+      <c r="AF81" s="315"/>
+      <c r="AG81" s="317"/>
       <c r="AL81" s="25"/>
       <c r="AM81" s="91"/>
     </row>
@@ -8353,9 +8353,9 @@
       <c r="D82" s="6"/>
       <c r="E82" s="6"/>
       <c r="F82" s="6"/>
-      <c r="G82" s="317"/>
-      <c r="H82" s="315"/>
-      <c r="I82" s="317"/>
+      <c r="G82" s="315"/>
+      <c r="H82" s="313"/>
+      <c r="I82" s="315"/>
       <c r="J82" s="31"/>
       <c r="K82" s="6"/>
       <c r="L82" s="6"/>
@@ -8365,7 +8365,7 @@
       <c r="Q82" s="104"/>
       <c r="R82" s="6"/>
       <c r="S82" s="6"/>
-      <c r="T82" s="317"/>
+      <c r="T82" s="315"/>
       <c r="U82" s="6"/>
       <c r="V82" s="6"/>
       <c r="W82" s="6"/>
@@ -8375,10 +8375,10 @@
       <c r="AA82" s="6"/>
       <c r="AB82" s="6"/>
       <c r="AC82" s="6"/>
-      <c r="AD82" s="317"/>
-      <c r="AE82" s="317"/>
-      <c r="AF82" s="317"/>
-      <c r="AG82" s="319"/>
+      <c r="AD82" s="315"/>
+      <c r="AE82" s="315"/>
+      <c r="AF82" s="315"/>
+      <c r="AG82" s="317"/>
       <c r="AL82" s="25"/>
       <c r="AM82" s="91"/>
     </row>
@@ -8388,9 +8388,9 @@
       <c r="D83" s="6"/>
       <c r="E83" s="6"/>
       <c r="F83" s="6"/>
-      <c r="G83" s="317"/>
-      <c r="H83" s="315"/>
-      <c r="I83" s="317"/>
+      <c r="G83" s="315"/>
+      <c r="H83" s="313"/>
+      <c r="I83" s="315"/>
       <c r="J83" s="31"/>
       <c r="K83" s="6"/>
       <c r="L83" s="6"/>
@@ -8410,10 +8410,10 @@
       <c r="AA83" s="6"/>
       <c r="AB83" s="6"/>
       <c r="AC83" s="6"/>
-      <c r="AD83" s="317"/>
-      <c r="AE83" s="317"/>
-      <c r="AF83" s="317"/>
-      <c r="AG83" s="319"/>
+      <c r="AD83" s="315"/>
+      <c r="AE83" s="315"/>
+      <c r="AF83" s="315"/>
+      <c r="AG83" s="317"/>
       <c r="AL83" s="25"/>
       <c r="AM83" s="91"/>
     </row>
@@ -8423,9 +8423,9 @@
       <c r="D84" s="6"/>
       <c r="E84" s="6"/>
       <c r="F84" s="6"/>
-      <c r="G84" s="317"/>
-      <c r="H84" s="315"/>
-      <c r="I84" s="317"/>
+      <c r="G84" s="315"/>
+      <c r="H84" s="313"/>
+      <c r="I84" s="315"/>
       <c r="J84" s="31"/>
       <c r="K84" s="6"/>
       <c r="L84" s="6"/>
@@ -8445,10 +8445,10 @@
       <c r="AA84" s="6"/>
       <c r="AB84" s="6"/>
       <c r="AC84" s="6"/>
-      <c r="AD84" s="317"/>
-      <c r="AE84" s="317"/>
-      <c r="AF84" s="317"/>
-      <c r="AG84" s="319"/>
+      <c r="AD84" s="315"/>
+      <c r="AE84" s="315"/>
+      <c r="AF84" s="315"/>
+      <c r="AG84" s="317"/>
       <c r="AL84" s="25"/>
       <c r="AM84" s="91"/>
     </row>
@@ -8458,9 +8458,9 @@
       <c r="D85" s="6"/>
       <c r="E85" s="6"/>
       <c r="F85" s="6"/>
-      <c r="G85" s="317"/>
-      <c r="H85" s="315"/>
-      <c r="I85" s="317"/>
+      <c r="G85" s="315"/>
+      <c r="H85" s="313"/>
+      <c r="I85" s="315"/>
       <c r="J85" s="31"/>
       <c r="K85" s="6"/>
       <c r="L85" s="6"/>
@@ -8480,10 +8480,10 @@
       <c r="AA85" s="6"/>
       <c r="AB85" s="6"/>
       <c r="AC85" s="6"/>
-      <c r="AD85" s="317"/>
-      <c r="AE85" s="317"/>
-      <c r="AF85" s="317"/>
-      <c r="AG85" s="319"/>
+      <c r="AD85" s="315"/>
+      <c r="AE85" s="315"/>
+      <c r="AF85" s="315"/>
+      <c r="AG85" s="317"/>
       <c r="AL85" s="25"/>
       <c r="AM85" s="91"/>
     </row>
@@ -8493,9 +8493,9 @@
       <c r="D86" s="6"/>
       <c r="E86" s="6"/>
       <c r="F86" s="6"/>
-      <c r="G86" s="317"/>
-      <c r="H86" s="315"/>
-      <c r="I86" s="317"/>
+      <c r="G86" s="315"/>
+      <c r="H86" s="313"/>
+      <c r="I86" s="315"/>
       <c r="J86" s="31"/>
       <c r="K86" s="6"/>
       <c r="L86" s="6"/>
@@ -8515,10 +8515,10 @@
       <c r="AA86" s="6"/>
       <c r="AB86" s="6"/>
       <c r="AC86" s="6"/>
-      <c r="AD86" s="317"/>
-      <c r="AE86" s="317"/>
-      <c r="AF86" s="317"/>
-      <c r="AG86" s="319"/>
+      <c r="AD86" s="315"/>
+      <c r="AE86" s="315"/>
+      <c r="AF86" s="315"/>
+      <c r="AG86" s="317"/>
       <c r="AL86" s="25"/>
       <c r="AM86" s="91"/>
     </row>
@@ -8528,9 +8528,9 @@
       <c r="D87" s="6"/>
       <c r="E87" s="6"/>
       <c r="F87" s="6"/>
-      <c r="G87" s="317"/>
-      <c r="H87" s="315"/>
-      <c r="I87" s="317"/>
+      <c r="G87" s="315"/>
+      <c r="H87" s="313"/>
+      <c r="I87" s="315"/>
       <c r="J87" s="31"/>
       <c r="K87" s="6"/>
       <c r="L87" s="6"/>
@@ -8550,10 +8550,10 @@
       <c r="AA87" s="6"/>
       <c r="AB87" s="6"/>
       <c r="AC87" s="6"/>
-      <c r="AD87" s="317"/>
-      <c r="AE87" s="317"/>
-      <c r="AF87" s="317"/>
-      <c r="AG87" s="319"/>
+      <c r="AD87" s="315"/>
+      <c r="AE87" s="315"/>
+      <c r="AF87" s="315"/>
+      <c r="AG87" s="317"/>
       <c r="AL87" s="25"/>
       <c r="AM87" s="91"/>
     </row>
@@ -8563,9 +8563,9 @@
       <c r="D88" s="6"/>
       <c r="E88" s="6"/>
       <c r="F88" s="6"/>
-      <c r="G88" s="317"/>
-      <c r="H88" s="315"/>
-      <c r="I88" s="317"/>
+      <c r="G88" s="315"/>
+      <c r="H88" s="313"/>
+      <c r="I88" s="315"/>
       <c r="J88" s="31"/>
       <c r="K88" s="6"/>
       <c r="L88" s="6"/>
@@ -8585,10 +8585,10 @@
       <c r="AA88" s="6"/>
       <c r="AB88" s="6"/>
       <c r="AC88" s="6"/>
-      <c r="AD88" s="317"/>
-      <c r="AE88" s="317"/>
-      <c r="AF88" s="317"/>
-      <c r="AG88" s="319"/>
+      <c r="AD88" s="315"/>
+      <c r="AE88" s="315"/>
+      <c r="AF88" s="315"/>
+      <c r="AG88" s="317"/>
       <c r="AL88" s="25"/>
       <c r="AM88" s="91"/>
     </row>
@@ -8620,10 +8620,10 @@
       <c r="AA89" s="6"/>
       <c r="AB89" s="6"/>
       <c r="AC89" s="6"/>
-      <c r="AD89" s="317"/>
-      <c r="AE89" s="317"/>
-      <c r="AF89" s="317"/>
-      <c r="AG89" s="319"/>
+      <c r="AD89" s="315"/>
+      <c r="AE89" s="315"/>
+      <c r="AF89" s="315"/>
+      <c r="AG89" s="317"/>
       <c r="AL89" s="25"/>
       <c r="AM89" s="91"/>
     </row>
@@ -8633,7 +8633,7 @@
       <c r="D90" s="6"/>
       <c r="E90" s="6"/>
       <c r="F90" s="6"/>
-      <c r="G90" s="317"/>
+      <c r="G90" s="315"/>
       <c r="H90" s="39"/>
       <c r="I90" s="6"/>
       <c r="J90" s="31"/>
@@ -8655,10 +8655,10 @@
       <c r="AA90" s="6"/>
       <c r="AB90" s="6"/>
       <c r="AC90" s="6"/>
-      <c r="AD90" s="317"/>
-      <c r="AE90" s="317"/>
-      <c r="AF90" s="317"/>
-      <c r="AG90" s="319"/>
+      <c r="AD90" s="315"/>
+      <c r="AE90" s="315"/>
+      <c r="AF90" s="315"/>
+      <c r="AG90" s="317"/>
       <c r="AL90" s="25"/>
       <c r="AM90" s="91"/>
     </row>
@@ -8668,9 +8668,9 @@
       <c r="D91" s="6"/>
       <c r="E91" s="6"/>
       <c r="F91" s="6"/>
-      <c r="G91" s="317"/>
-      <c r="H91" s="315"/>
-      <c r="I91" s="317"/>
+      <c r="G91" s="315"/>
+      <c r="H91" s="313"/>
+      <c r="I91" s="315"/>
       <c r="J91" s="31"/>
       <c r="K91" s="6"/>
       <c r="L91" s="6"/>
@@ -8690,10 +8690,10 @@
       <c r="AA91" s="6"/>
       <c r="AB91" s="6"/>
       <c r="AC91" s="6"/>
-      <c r="AD91" s="317"/>
-      <c r="AE91" s="317"/>
-      <c r="AF91" s="317"/>
-      <c r="AG91" s="319"/>
+      <c r="AD91" s="315"/>
+      <c r="AE91" s="315"/>
+      <c r="AF91" s="315"/>
+      <c r="AG91" s="317"/>
       <c r="AL91" s="25"/>
       <c r="AM91" s="91"/>
     </row>
@@ -8703,9 +8703,9 @@
       <c r="D92" s="6"/>
       <c r="E92" s="6"/>
       <c r="F92" s="6"/>
-      <c r="G92" s="317"/>
-      <c r="H92" s="315"/>
-      <c r="I92" s="317"/>
+      <c r="G92" s="315"/>
+      <c r="H92" s="313"/>
+      <c r="I92" s="315"/>
       <c r="J92" s="31"/>
       <c r="K92" s="6"/>
       <c r="L92" s="6"/>
@@ -8725,10 +8725,10 @@
       <c r="AA92" s="6"/>
       <c r="AB92" s="6"/>
       <c r="AC92" s="6"/>
-      <c r="AD92" s="317"/>
-      <c r="AE92" s="317"/>
-      <c r="AF92" s="317"/>
-      <c r="AG92" s="319"/>
+      <c r="AD92" s="315"/>
+      <c r="AE92" s="315"/>
+      <c r="AF92" s="315"/>
+      <c r="AG92" s="317"/>
       <c r="AL92" s="25"/>
       <c r="AM92" s="91"/>
     </row>
@@ -8738,9 +8738,9 @@
       <c r="D93" s="6"/>
       <c r="E93" s="6"/>
       <c r="F93" s="6"/>
-      <c r="G93" s="317"/>
-      <c r="H93" s="315"/>
-      <c r="I93" s="317"/>
+      <c r="G93" s="315"/>
+      <c r="H93" s="313"/>
+      <c r="I93" s="315"/>
       <c r="J93" s="31"/>
       <c r="K93" s="6"/>
       <c r="L93" s="6"/>
@@ -8760,10 +8760,10 @@
       <c r="AA93" s="6"/>
       <c r="AB93" s="6"/>
       <c r="AC93" s="6"/>
-      <c r="AD93" s="317"/>
-      <c r="AE93" s="317"/>
-      <c r="AF93" s="317"/>
-      <c r="AG93" s="319"/>
+      <c r="AD93" s="315"/>
+      <c r="AE93" s="315"/>
+      <c r="AF93" s="315"/>
+      <c r="AG93" s="317"/>
       <c r="AL93" s="25"/>
       <c r="AM93" s="91"/>
     </row>
@@ -8773,9 +8773,9 @@
       <c r="D94" s="6"/>
       <c r="E94" s="6"/>
       <c r="F94" s="6"/>
-      <c r="G94" s="317"/>
-      <c r="H94" s="315"/>
-      <c r="I94" s="317"/>
+      <c r="G94" s="315"/>
+      <c r="H94" s="313"/>
+      <c r="I94" s="315"/>
       <c r="J94" s="31"/>
       <c r="K94" s="6"/>
       <c r="L94" s="6"/>
@@ -8795,10 +8795,10 @@
       <c r="AA94" s="6"/>
       <c r="AB94" s="6"/>
       <c r="AC94" s="6"/>
-      <c r="AD94" s="317"/>
-      <c r="AE94" s="317"/>
-      <c r="AF94" s="317"/>
-      <c r="AG94" s="319"/>
+      <c r="AD94" s="315"/>
+      <c r="AE94" s="315"/>
+      <c r="AF94" s="315"/>
+      <c r="AG94" s="317"/>
       <c r="AL94" s="25"/>
       <c r="AM94" s="91"/>
     </row>
@@ -8808,9 +8808,9 @@
       <c r="D95" s="6"/>
       <c r="E95" s="6"/>
       <c r="F95" s="6"/>
-      <c r="G95" s="317"/>
-      <c r="H95" s="315"/>
-      <c r="I95" s="317"/>
+      <c r="G95" s="315"/>
+      <c r="H95" s="313"/>
+      <c r="I95" s="315"/>
       <c r="J95" s="31"/>
       <c r="K95" s="6"/>
       <c r="L95" s="6"/>
@@ -8830,10 +8830,10 @@
       <c r="AA95" s="6"/>
       <c r="AB95" s="6"/>
       <c r="AC95" s="6"/>
-      <c r="AD95" s="317"/>
-      <c r="AE95" s="317"/>
-      <c r="AF95" s="317"/>
-      <c r="AG95" s="319"/>
+      <c r="AD95" s="315"/>
+      <c r="AE95" s="315"/>
+      <c r="AF95" s="315"/>
+      <c r="AG95" s="317"/>
       <c r="AL95" s="25"/>
       <c r="AM95" s="91"/>
     </row>
@@ -8843,9 +8843,9 @@
       <c r="D96" s="6"/>
       <c r="E96" s="6"/>
       <c r="F96" s="6"/>
-      <c r="G96" s="317"/>
-      <c r="H96" s="315"/>
-      <c r="I96" s="317"/>
+      <c r="G96" s="315"/>
+      <c r="H96" s="313"/>
+      <c r="I96" s="315"/>
       <c r="J96" s="31"/>
       <c r="K96" s="6"/>
       <c r="L96" s="6"/>
@@ -8865,10 +8865,10 @@
       <c r="AA96" s="6"/>
       <c r="AB96" s="6"/>
       <c r="AC96" s="6"/>
-      <c r="AD96" s="317"/>
-      <c r="AE96" s="317"/>
-      <c r="AF96" s="317"/>
-      <c r="AG96" s="319"/>
+      <c r="AD96" s="315"/>
+      <c r="AE96" s="315"/>
+      <c r="AF96" s="315"/>
+      <c r="AG96" s="317"/>
       <c r="AL96" s="25"/>
       <c r="AM96" s="91"/>
     </row>
@@ -8878,9 +8878,9 @@
       <c r="D97" s="6"/>
       <c r="E97" s="6"/>
       <c r="F97" s="6"/>
-      <c r="G97" s="317"/>
-      <c r="H97" s="315"/>
-      <c r="I97" s="317"/>
+      <c r="G97" s="315"/>
+      <c r="H97" s="313"/>
+      <c r="I97" s="315"/>
       <c r="J97" s="31"/>
       <c r="K97" s="6"/>
       <c r="L97" s="6"/>
@@ -8900,10 +8900,10 @@
       <c r="AA97" s="6"/>
       <c r="AB97" s="6"/>
       <c r="AC97" s="6"/>
-      <c r="AD97" s="317"/>
-      <c r="AE97" s="317"/>
-      <c r="AF97" s="317"/>
-      <c r="AG97" s="319"/>
+      <c r="AD97" s="315"/>
+      <c r="AE97" s="315"/>
+      <c r="AF97" s="315"/>
+      <c r="AG97" s="317"/>
       <c r="AL97" s="25"/>
       <c r="AM97" s="91"/>
     </row>
@@ -8913,9 +8913,9 @@
       <c r="D98" s="6"/>
       <c r="E98" s="6"/>
       <c r="F98" s="6"/>
-      <c r="G98" s="317"/>
-      <c r="H98" s="315"/>
-      <c r="I98" s="317"/>
+      <c r="G98" s="315"/>
+      <c r="H98" s="313"/>
+      <c r="I98" s="315"/>
       <c r="J98" s="31"/>
       <c r="K98" s="6"/>
       <c r="L98" s="6"/>
@@ -8935,10 +8935,10 @@
       <c r="AA98" s="6"/>
       <c r="AB98" s="6"/>
       <c r="AC98" s="6"/>
-      <c r="AD98" s="317"/>
-      <c r="AE98" s="317"/>
-      <c r="AF98" s="317"/>
-      <c r="AG98" s="319"/>
+      <c r="AD98" s="315"/>
+      <c r="AE98" s="315"/>
+      <c r="AF98" s="315"/>
+      <c r="AG98" s="317"/>
       <c r="AL98" s="25"/>
       <c r="AM98" s="91"/>
     </row>
@@ -8948,9 +8948,9 @@
       <c r="D99" s="6"/>
       <c r="E99" s="6"/>
       <c r="F99" s="6"/>
-      <c r="G99" s="317"/>
-      <c r="H99" s="315"/>
-      <c r="I99" s="317"/>
+      <c r="G99" s="315"/>
+      <c r="H99" s="313"/>
+      <c r="I99" s="315"/>
       <c r="J99" s="31"/>
       <c r="K99" s="6"/>
       <c r="L99" s="6"/>
@@ -8970,10 +8970,10 @@
       <c r="AA99" s="6"/>
       <c r="AB99" s="6"/>
       <c r="AC99" s="6"/>
-      <c r="AD99" s="317"/>
-      <c r="AE99" s="317"/>
-      <c r="AF99" s="317"/>
-      <c r="AG99" s="319"/>
+      <c r="AD99" s="315"/>
+      <c r="AE99" s="315"/>
+      <c r="AF99" s="315"/>
+      <c r="AG99" s="317"/>
       <c r="AL99" s="25"/>
       <c r="AM99" s="91"/>
     </row>
@@ -8983,9 +8983,9 @@
       <c r="D100" s="6"/>
       <c r="E100" s="6"/>
       <c r="F100" s="6"/>
-      <c r="G100" s="317"/>
-      <c r="H100" s="315"/>
-      <c r="I100" s="317"/>
+      <c r="G100" s="315"/>
+      <c r="H100" s="313"/>
+      <c r="I100" s="315"/>
       <c r="J100" s="31"/>
       <c r="K100" s="6"/>
       <c r="L100" s="6"/>
@@ -9005,10 +9005,10 @@
       <c r="AA100" s="6"/>
       <c r="AB100" s="6"/>
       <c r="AC100" s="6"/>
-      <c r="AD100" s="317"/>
-      <c r="AE100" s="317"/>
-      <c r="AF100" s="317"/>
-      <c r="AG100" s="319"/>
+      <c r="AD100" s="315"/>
+      <c r="AE100" s="315"/>
+      <c r="AF100" s="315"/>
+      <c r="AG100" s="317"/>
       <c r="AL100" s="25"/>
       <c r="AM100" s="91"/>
     </row>
@@ -9018,9 +9018,9 @@
       <c r="D101" s="6"/>
       <c r="E101" s="6"/>
       <c r="F101" s="6"/>
-      <c r="G101" s="317"/>
-      <c r="H101" s="315"/>
-      <c r="I101" s="317"/>
+      <c r="G101" s="315"/>
+      <c r="H101" s="313"/>
+      <c r="I101" s="315"/>
       <c r="J101" s="31"/>
       <c r="K101" s="6"/>
       <c r="L101" s="6"/>
@@ -9040,10 +9040,10 @@
       <c r="AA101" s="6"/>
       <c r="AB101" s="6"/>
       <c r="AC101" s="6"/>
-      <c r="AD101" s="317"/>
-      <c r="AE101" s="317"/>
-      <c r="AF101" s="317"/>
-      <c r="AG101" s="319"/>
+      <c r="AD101" s="315"/>
+      <c r="AE101" s="315"/>
+      <c r="AF101" s="315"/>
+      <c r="AG101" s="317"/>
       <c r="AL101" s="25"/>
       <c r="AM101" s="91"/>
     </row>
@@ -9053,9 +9053,9 @@
       <c r="D102" s="6"/>
       <c r="E102" s="6"/>
       <c r="F102" s="6"/>
-      <c r="G102" s="317"/>
-      <c r="H102" s="315"/>
-      <c r="I102" s="317"/>
+      <c r="G102" s="315"/>
+      <c r="H102" s="313"/>
+      <c r="I102" s="315"/>
       <c r="J102" s="31"/>
       <c r="K102" s="6"/>
       <c r="L102" s="6"/>
@@ -9075,10 +9075,10 @@
       <c r="AA102" s="6"/>
       <c r="AB102" s="6"/>
       <c r="AC102" s="6"/>
-      <c r="AD102" s="317"/>
-      <c r="AE102" s="317"/>
-      <c r="AF102" s="317"/>
-      <c r="AG102" s="319"/>
+      <c r="AD102" s="315"/>
+      <c r="AE102" s="315"/>
+      <c r="AF102" s="315"/>
+      <c r="AG102" s="317"/>
       <c r="AL102" s="25"/>
       <c r="AM102" s="91"/>
     </row>
@@ -9088,9 +9088,9 @@
       <c r="D103" s="6"/>
       <c r="E103" s="6"/>
       <c r="F103" s="6"/>
-      <c r="G103" s="317"/>
-      <c r="H103" s="315"/>
-      <c r="I103" s="317"/>
+      <c r="G103" s="315"/>
+      <c r="H103" s="313"/>
+      <c r="I103" s="315"/>
       <c r="J103" s="31"/>
       <c r="K103" s="6"/>
       <c r="L103" s="6"/>
@@ -9110,10 +9110,10 @@
       <c r="AA103" s="6"/>
       <c r="AB103" s="6"/>
       <c r="AC103" s="6"/>
-      <c r="AD103" s="317"/>
-      <c r="AE103" s="317"/>
-      <c r="AF103" s="317"/>
-      <c r="AG103" s="319"/>
+      <c r="AD103" s="315"/>
+      <c r="AE103" s="315"/>
+      <c r="AF103" s="315"/>
+      <c r="AG103" s="317"/>
       <c r="AL103" s="25"/>
       <c r="AM103" s="91"/>
     </row>
@@ -9123,9 +9123,9 @@
       <c r="D104" s="6"/>
       <c r="E104" s="6"/>
       <c r="F104" s="6"/>
-      <c r="G104" s="317"/>
-      <c r="H104" s="315"/>
-      <c r="I104" s="317"/>
+      <c r="G104" s="315"/>
+      <c r="H104" s="313"/>
+      <c r="I104" s="315"/>
       <c r="J104" s="31"/>
       <c r="K104" s="6"/>
       <c r="L104" s="6"/>
@@ -9145,10 +9145,10 @@
       <c r="AA104" s="6"/>
       <c r="AB104" s="6"/>
       <c r="AC104" s="6"/>
-      <c r="AD104" s="317"/>
-      <c r="AE104" s="317"/>
-      <c r="AF104" s="317"/>
-      <c r="AG104" s="319"/>
+      <c r="AD104" s="315"/>
+      <c r="AE104" s="315"/>
+      <c r="AF104" s="315"/>
+      <c r="AG104" s="317"/>
       <c r="AL104" s="25"/>
       <c r="AM104" s="91"/>
     </row>
@@ -9158,9 +9158,9 @@
       <c r="D105" s="6"/>
       <c r="E105" s="6"/>
       <c r="F105" s="6"/>
-      <c r="G105" s="317"/>
-      <c r="H105" s="315"/>
-      <c r="I105" s="317"/>
+      <c r="G105" s="315"/>
+      <c r="H105" s="313"/>
+      <c r="I105" s="315"/>
       <c r="J105" s="31"/>
       <c r="K105" s="6"/>
       <c r="L105" s="6"/>
@@ -9180,10 +9180,10 @@
       <c r="AA105" s="6"/>
       <c r="AB105" s="6"/>
       <c r="AC105" s="6"/>
-      <c r="AD105" s="317"/>
-      <c r="AE105" s="317"/>
-      <c r="AF105" s="317"/>
-      <c r="AG105" s="319"/>
+      <c r="AD105" s="315"/>
+      <c r="AE105" s="315"/>
+      <c r="AF105" s="315"/>
+      <c r="AG105" s="317"/>
       <c r="AL105" s="25"/>
       <c r="AM105" s="91"/>
     </row>
@@ -9193,9 +9193,9 @@
       <c r="D106" s="140"/>
       <c r="E106" s="140"/>
       <c r="F106" s="140"/>
-      <c r="G106" s="320"/>
-      <c r="H106" s="321"/>
-      <c r="I106" s="320"/>
+      <c r="G106" s="318"/>
+      <c r="H106" s="319"/>
+      <c r="I106" s="318"/>
       <c r="J106" s="6"/>
       <c r="K106" s="6"/>
       <c r="L106" s="6"/>
@@ -9215,10 +9215,10 @@
       <c r="AA106" s="6"/>
       <c r="AB106" s="6"/>
       <c r="AC106" s="6"/>
-      <c r="AD106" s="317"/>
-      <c r="AE106" s="317"/>
-      <c r="AF106" s="317"/>
-      <c r="AG106" s="319"/>
+      <c r="AD106" s="315"/>
+      <c r="AE106" s="315"/>
+      <c r="AF106" s="315"/>
+      <c r="AG106" s="317"/>
       <c r="AL106" s="25"/>
       <c r="AM106" s="91"/>
     </row>
@@ -9228,9 +9228,9 @@
       <c r="D107" s="6"/>
       <c r="E107" s="6"/>
       <c r="F107" s="6"/>
-      <c r="G107" s="317"/>
-      <c r="H107" s="315"/>
-      <c r="I107" s="317"/>
+      <c r="G107" s="315"/>
+      <c r="H107" s="313"/>
+      <c r="I107" s="315"/>
       <c r="J107" s="6"/>
       <c r="K107" s="6"/>
       <c r="L107" s="6"/>
@@ -9250,10 +9250,10 @@
       <c r="AA107" s="6"/>
       <c r="AB107" s="6"/>
       <c r="AC107" s="6"/>
-      <c r="AD107" s="317"/>
-      <c r="AE107" s="317"/>
-      <c r="AF107" s="317"/>
-      <c r="AG107" s="319"/>
+      <c r="AD107" s="315"/>
+      <c r="AE107" s="315"/>
+      <c r="AF107" s="315"/>
+      <c r="AG107" s="317"/>
       <c r="AL107" s="25"/>
       <c r="AM107" s="91"/>
     </row>
@@ -9263,9 +9263,9 @@
       <c r="D108" s="6"/>
       <c r="E108" s="6"/>
       <c r="F108" s="6"/>
-      <c r="G108" s="317"/>
-      <c r="H108" s="315"/>
-      <c r="I108" s="317"/>
+      <c r="G108" s="315"/>
+      <c r="H108" s="313"/>
+      <c r="I108" s="315"/>
       <c r="J108" s="6"/>
       <c r="K108" s="6"/>
       <c r="L108" s="6"/>
@@ -9285,10 +9285,10 @@
       <c r="AA108" s="6"/>
       <c r="AB108" s="6"/>
       <c r="AC108" s="6"/>
-      <c r="AD108" s="317"/>
-      <c r="AE108" s="317"/>
-      <c r="AF108" s="317"/>
-      <c r="AG108" s="319"/>
+      <c r="AD108" s="315"/>
+      <c r="AE108" s="315"/>
+      <c r="AF108" s="315"/>
+      <c r="AG108" s="317"/>
       <c r="AL108" s="25"/>
       <c r="AM108" s="91"/>
     </row>
@@ -9298,9 +9298,9 @@
       <c r="D109" s="6"/>
       <c r="E109" s="6"/>
       <c r="F109" s="6"/>
-      <c r="G109" s="317"/>
-      <c r="H109" s="315"/>
-      <c r="I109" s="317"/>
+      <c r="G109" s="315"/>
+      <c r="H109" s="313"/>
+      <c r="I109" s="315"/>
       <c r="J109" s="6"/>
       <c r="K109" s="6"/>
       <c r="L109" s="6"/>
@@ -9320,10 +9320,10 @@
       <c r="AA109" s="6"/>
       <c r="AB109" s="6"/>
       <c r="AC109" s="6"/>
-      <c r="AD109" s="317"/>
-      <c r="AE109" s="317"/>
-      <c r="AF109" s="317"/>
-      <c r="AG109" s="319"/>
+      <c r="AD109" s="315"/>
+      <c r="AE109" s="315"/>
+      <c r="AF109" s="315"/>
+      <c r="AG109" s="317"/>
       <c r="AL109" s="25"/>
       <c r="AM109" s="91"/>
     </row>
@@ -9333,9 +9333,9 @@
       <c r="D110" s="6"/>
       <c r="E110" s="6"/>
       <c r="F110" s="6"/>
-      <c r="G110" s="317"/>
-      <c r="H110" s="315"/>
-      <c r="I110" s="317"/>
+      <c r="G110" s="315"/>
+      <c r="H110" s="313"/>
+      <c r="I110" s="315"/>
       <c r="J110" s="6"/>
       <c r="K110" s="6"/>
       <c r="L110" s="6"/>
@@ -9355,10 +9355,10 @@
       <c r="AA110" s="6"/>
       <c r="AB110" s="6"/>
       <c r="AC110" s="6"/>
-      <c r="AD110" s="317"/>
-      <c r="AE110" s="317"/>
-      <c r="AF110" s="317"/>
-      <c r="AG110" s="319"/>
+      <c r="AD110" s="315"/>
+      <c r="AE110" s="315"/>
+      <c r="AF110" s="315"/>
+      <c r="AG110" s="317"/>
       <c r="AL110" s="25"/>
       <c r="AM110" s="91"/>
     </row>
@@ -9368,9 +9368,9 @@
       <c r="D111" s="6"/>
       <c r="E111" s="6"/>
       <c r="F111" s="6"/>
-      <c r="G111" s="317"/>
-      <c r="H111" s="315"/>
-      <c r="I111" s="317"/>
+      <c r="G111" s="315"/>
+      <c r="H111" s="313"/>
+      <c r="I111" s="315"/>
       <c r="J111" s="6"/>
       <c r="K111" s="6"/>
       <c r="L111" s="6"/>
@@ -9390,10 +9390,10 @@
       <c r="AA111" s="6"/>
       <c r="AB111" s="6"/>
       <c r="AC111" s="6"/>
-      <c r="AD111" s="317"/>
-      <c r="AE111" s="317"/>
-      <c r="AF111" s="317"/>
-      <c r="AG111" s="319"/>
+      <c r="AD111" s="315"/>
+      <c r="AE111" s="315"/>
+      <c r="AF111" s="315"/>
+      <c r="AG111" s="317"/>
       <c r="AL111" s="25"/>
       <c r="AM111" s="91"/>
     </row>
@@ -9403,9 +9403,9 @@
       <c r="D112" s="6"/>
       <c r="E112" s="6"/>
       <c r="F112" s="6"/>
-      <c r="G112" s="317"/>
-      <c r="H112" s="315"/>
-      <c r="I112" s="317"/>
+      <c r="G112" s="315"/>
+      <c r="H112" s="313"/>
+      <c r="I112" s="315"/>
       <c r="J112" s="6"/>
       <c r="K112" s="6"/>
       <c r="L112" s="6"/>
@@ -9438,9 +9438,9 @@
       <c r="D113" s="6"/>
       <c r="E113" s="6"/>
       <c r="F113" s="6"/>
-      <c r="G113" s="317"/>
-      <c r="H113" s="315"/>
-      <c r="I113" s="317"/>
+      <c r="G113" s="315"/>
+      <c r="H113" s="313"/>
+      <c r="I113" s="315"/>
       <c r="J113" s="6"/>
       <c r="K113" s="6"/>
       <c r="L113" s="6"/>
@@ -9473,9 +9473,9 @@
       <c r="D114" s="6"/>
       <c r="E114" s="6"/>
       <c r="F114" s="6"/>
-      <c r="G114" s="317"/>
-      <c r="H114" s="315"/>
-      <c r="I114" s="317"/>
+      <c r="G114" s="315"/>
+      <c r="H114" s="313"/>
+      <c r="I114" s="315"/>
       <c r="J114" s="6"/>
       <c r="K114" s="6"/>
       <c r="L114" s="6"/>
@@ -9508,9 +9508,9 @@
       <c r="D115" s="6"/>
       <c r="E115" s="6"/>
       <c r="F115" s="6"/>
-      <c r="G115" s="317"/>
-      <c r="H115" s="315"/>
-      <c r="I115" s="317"/>
+      <c r="G115" s="315"/>
+      <c r="H115" s="313"/>
+      <c r="I115" s="315"/>
       <c r="J115" s="6"/>
       <c r="K115" s="6"/>
       <c r="L115" s="6"/>
@@ -9543,9 +9543,9 @@
       <c r="D116" s="6"/>
       <c r="E116" s="6"/>
       <c r="F116" s="6"/>
-      <c r="G116" s="317"/>
-      <c r="H116" s="315"/>
-      <c r="I116" s="317"/>
+      <c r="G116" s="315"/>
+      <c r="H116" s="313"/>
+      <c r="I116" s="315"/>
       <c r="J116" s="6"/>
       <c r="K116" s="6"/>
       <c r="L116" s="6"/>
@@ -9579,8 +9579,8 @@
       <c r="E117" s="6"/>
       <c r="F117" s="6"/>
       <c r="G117" s="6"/>
-      <c r="H117" s="315"/>
-      <c r="I117" s="317"/>
+      <c r="H117" s="313"/>
+      <c r="I117" s="315"/>
       <c r="J117" s="6"/>
       <c r="K117" s="6"/>
       <c r="L117" s="6"/>
@@ -9614,8 +9614,8 @@
       <c r="E118" s="6"/>
       <c r="F118" s="6"/>
       <c r="G118" s="6"/>
-      <c r="H118" s="315"/>
-      <c r="I118" s="317"/>
+      <c r="H118" s="313"/>
+      <c r="I118" s="315"/>
       <c r="J118" s="6"/>
       <c r="K118" s="6"/>
       <c r="L118" s="6"/>
@@ -9649,8 +9649,8 @@
       <c r="E119" s="6"/>
       <c r="F119" s="6"/>
       <c r="G119" s="6"/>
-      <c r="H119" s="315"/>
-      <c r="I119" s="317"/>
+      <c r="H119" s="313"/>
+      <c r="I119" s="315"/>
       <c r="J119" s="6"/>
       <c r="K119" s="6"/>
       <c r="L119" s="6"/>
@@ -9684,8 +9684,8 @@
       <c r="E120" s="6"/>
       <c r="F120" s="6"/>
       <c r="G120" s="6"/>
-      <c r="H120" s="315"/>
-      <c r="I120" s="317"/>
+      <c r="H120" s="313"/>
+      <c r="I120" s="315"/>
       <c r="J120" s="6"/>
       <c r="K120" s="6"/>
       <c r="L120" s="6"/>
@@ -9719,8 +9719,8 @@
       <c r="E121" s="6"/>
       <c r="F121" s="6"/>
       <c r="G121" s="6"/>
-      <c r="H121" s="315"/>
-      <c r="I121" s="317"/>
+      <c r="H121" s="313"/>
+      <c r="I121" s="315"/>
       <c r="J121" s="6"/>
       <c r="K121" s="6"/>
       <c r="L121" s="6"/>
@@ -9754,8 +9754,8 @@
       <c r="E122" s="6"/>
       <c r="F122" s="6"/>
       <c r="G122" s="6"/>
-      <c r="H122" s="315"/>
-      <c r="I122" s="317"/>
+      <c r="H122" s="313"/>
+      <c r="I122" s="315"/>
       <c r="J122" s="6"/>
       <c r="K122" s="6"/>
       <c r="L122" s="6"/>
@@ -9789,8 +9789,8 @@
       <c r="E123" s="6"/>
       <c r="F123" s="6"/>
       <c r="G123" s="6"/>
-      <c r="H123" s="315"/>
-      <c r="I123" s="317"/>
+      <c r="H123" s="313"/>
+      <c r="I123" s="315"/>
       <c r="J123" s="6"/>
       <c r="K123" s="6"/>
       <c r="L123" s="6"/>
@@ -9824,8 +9824,8 @@
       <c r="E124" s="6"/>
       <c r="F124" s="6"/>
       <c r="G124" s="6"/>
-      <c r="H124" s="315"/>
-      <c r="I124" s="317"/>
+      <c r="H124" s="313"/>
+      <c r="I124" s="315"/>
       <c r="J124" s="6"/>
       <c r="K124" s="6"/>
       <c r="L124" s="6"/>
@@ -9859,8 +9859,8 @@
       <c r="E125" s="6"/>
       <c r="F125" s="6"/>
       <c r="G125" s="6"/>
-      <c r="H125" s="315"/>
-      <c r="I125" s="317"/>
+      <c r="H125" s="313"/>
+      <c r="I125" s="315"/>
       <c r="J125" s="6"/>
       <c r="K125" s="6"/>
       <c r="L125" s="6"/>
@@ -9894,8 +9894,8 @@
       <c r="E126" s="6"/>
       <c r="F126" s="6"/>
       <c r="G126" s="6"/>
-      <c r="H126" s="315"/>
-      <c r="I126" s="317"/>
+      <c r="H126" s="313"/>
+      <c r="I126" s="315"/>
       <c r="J126" s="6"/>
       <c r="K126" s="6"/>
       <c r="L126" s="6"/>
@@ -9929,8 +9929,8 @@
       <c r="E127" s="6"/>
       <c r="F127" s="6"/>
       <c r="G127" s="6"/>
-      <c r="H127" s="315"/>
-      <c r="I127" s="317"/>
+      <c r="H127" s="313"/>
+      <c r="I127" s="315"/>
       <c r="J127" s="6"/>
       <c r="K127" s="6"/>
       <c r="L127" s="6"/>
@@ -9964,8 +9964,8 @@
       <c r="E128" s="6"/>
       <c r="F128" s="6"/>
       <c r="G128" s="6"/>
-      <c r="H128" s="315"/>
-      <c r="I128" s="317"/>
+      <c r="H128" s="313"/>
+      <c r="I128" s="315"/>
       <c r="J128" s="6"/>
       <c r="K128" s="6"/>
       <c r="L128" s="6"/>
@@ -9999,8 +9999,8 @@
       <c r="E129" s="6"/>
       <c r="F129" s="6"/>
       <c r="G129" s="6"/>
-      <c r="H129" s="315"/>
-      <c r="I129" s="317"/>
+      <c r="H129" s="313"/>
+      <c r="I129" s="315"/>
       <c r="J129" s="6"/>
       <c r="K129" s="6"/>
       <c r="L129" s="6"/>
@@ -10034,8 +10034,8 @@
       <c r="E130" s="6"/>
       <c r="F130" s="6"/>
       <c r="G130" s="6"/>
-      <c r="H130" s="315"/>
-      <c r="I130" s="317"/>
+      <c r="H130" s="313"/>
+      <c r="I130" s="315"/>
       <c r="J130" s="6"/>
       <c r="K130" s="6"/>
       <c r="L130" s="6"/>
@@ -10069,8 +10069,8 @@
       <c r="E131" s="6"/>
       <c r="F131" s="6"/>
       <c r="G131" s="6"/>
-      <c r="H131" s="315"/>
-      <c r="I131" s="317"/>
+      <c r="H131" s="313"/>
+      <c r="I131" s="315"/>
       <c r="J131" s="6"/>
       <c r="K131" s="6"/>
       <c r="L131" s="6"/>
@@ -10104,8 +10104,8 @@
       <c r="E132" s="6"/>
       <c r="F132" s="6"/>
       <c r="G132" s="6"/>
-      <c r="H132" s="315"/>
-      <c r="I132" s="317"/>
+      <c r="H132" s="313"/>
+      <c r="I132" s="315"/>
       <c r="J132" s="6"/>
       <c r="K132" s="6"/>
       <c r="L132" s="6"/>
@@ -10139,8 +10139,8 @@
       <c r="E133" s="6"/>
       <c r="F133" s="6"/>
       <c r="G133" s="6"/>
-      <c r="H133" s="315"/>
-      <c r="I133" s="317"/>
+      <c r="H133" s="313"/>
+      <c r="I133" s="315"/>
       <c r="J133" s="6"/>
       <c r="K133" s="6"/>
       <c r="L133" s="6"/>
@@ -10174,8 +10174,8 @@
       <c r="E134" s="6"/>
       <c r="F134" s="6"/>
       <c r="G134" s="6"/>
-      <c r="H134" s="315"/>
-      <c r="I134" s="317"/>
+      <c r="H134" s="313"/>
+      <c r="I134" s="315"/>
       <c r="J134" s="6"/>
       <c r="K134" s="6"/>
       <c r="L134" s="6"/>
@@ -10209,8 +10209,8 @@
       <c r="E135" s="6"/>
       <c r="F135" s="6"/>
       <c r="G135" s="6"/>
-      <c r="H135" s="315"/>
-      <c r="I135" s="317"/>
+      <c r="H135" s="313"/>
+      <c r="I135" s="315"/>
       <c r="J135" s="6"/>
       <c r="K135" s="6"/>
       <c r="L135" s="6"/>
@@ -10244,8 +10244,8 @@
       <c r="E136" s="6"/>
       <c r="F136" s="6"/>
       <c r="G136" s="6"/>
-      <c r="H136" s="315"/>
-      <c r="I136" s="317"/>
+      <c r="H136" s="313"/>
+      <c r="I136" s="315"/>
       <c r="J136" s="6"/>
       <c r="K136" s="6"/>
       <c r="L136" s="6"/>
@@ -10279,8 +10279,8 @@
       <c r="E137" s="6"/>
       <c r="F137" s="6"/>
       <c r="G137" s="6"/>
-      <c r="H137" s="315"/>
-      <c r="I137" s="317"/>
+      <c r="H137" s="313"/>
+      <c r="I137" s="315"/>
       <c r="J137" s="6"/>
       <c r="K137" s="6"/>
       <c r="L137" s="6"/>
@@ -10314,8 +10314,8 @@
       <c r="E138" s="6"/>
       <c r="F138" s="6"/>
       <c r="G138" s="6"/>
-      <c r="H138" s="315"/>
-      <c r="I138" s="317"/>
+      <c r="H138" s="313"/>
+      <c r="I138" s="315"/>
       <c r="J138" s="6"/>
       <c r="K138" s="6"/>
       <c r="L138" s="6"/>
@@ -10349,8 +10349,8 @@
       <c r="E139" s="6"/>
       <c r="F139" s="6"/>
       <c r="G139" s="6"/>
-      <c r="H139" s="315"/>
-      <c r="I139" s="317"/>
+      <c r="H139" s="313"/>
+      <c r="I139" s="315"/>
       <c r="J139" s="6"/>
       <c r="K139" s="6"/>
       <c r="L139" s="6"/>
@@ -10384,8 +10384,8 @@
       <c r="E140" s="6"/>
       <c r="F140" s="6"/>
       <c r="G140" s="6"/>
-      <c r="H140" s="315"/>
-      <c r="I140" s="317"/>
+      <c r="H140" s="313"/>
+      <c r="I140" s="315"/>
       <c r="J140" s="6"/>
       <c r="K140" s="6"/>
       <c r="L140" s="6"/>
@@ -10419,8 +10419,8 @@
       <c r="E141" s="6"/>
       <c r="F141" s="6"/>
       <c r="G141" s="6"/>
-      <c r="H141" s="315"/>
-      <c r="I141" s="317"/>
+      <c r="H141" s="313"/>
+      <c r="I141" s="315"/>
       <c r="J141" s="6"/>
       <c r="K141" s="6"/>
       <c r="L141" s="6"/>
@@ -10454,8 +10454,8 @@
       <c r="E142" s="6"/>
       <c r="F142" s="6"/>
       <c r="G142" s="6"/>
-      <c r="H142" s="315"/>
-      <c r="I142" s="317"/>
+      <c r="H142" s="313"/>
+      <c r="I142" s="315"/>
       <c r="J142" s="6"/>
       <c r="K142" s="6"/>
       <c r="L142" s="6"/>
@@ -10489,8 +10489,8 @@
       <c r="E143" s="6"/>
       <c r="F143" s="6"/>
       <c r="G143" s="6"/>
-      <c r="H143" s="315"/>
-      <c r="I143" s="317"/>
+      <c r="H143" s="313"/>
+      <c r="I143" s="315"/>
       <c r="J143" s="6"/>
       <c r="K143" s="6"/>
       <c r="L143" s="6"/>
@@ -10524,8 +10524,8 @@
       <c r="E144" s="6"/>
       <c r="F144" s="6"/>
       <c r="G144" s="6"/>
-      <c r="H144" s="315"/>
-      <c r="I144" s="317"/>
+      <c r="H144" s="313"/>
+      <c r="I144" s="315"/>
       <c r="J144" s="6"/>
       <c r="K144" s="6"/>
       <c r="L144" s="6"/>
@@ -10559,8 +10559,8 @@
       <c r="E145" s="6"/>
       <c r="F145" s="6"/>
       <c r="G145" s="6"/>
-      <c r="H145" s="315"/>
-      <c r="I145" s="317"/>
+      <c r="H145" s="313"/>
+      <c r="I145" s="315"/>
       <c r="J145" s="6"/>
       <c r="K145" s="6"/>
       <c r="L145" s="6"/>
@@ -10594,8 +10594,8 @@
       <c r="E146" s="6"/>
       <c r="F146" s="6"/>
       <c r="G146" s="6"/>
-      <c r="H146" s="315"/>
-      <c r="I146" s="317"/>
+      <c r="H146" s="313"/>
+      <c r="I146" s="315"/>
       <c r="J146" s="6"/>
       <c r="K146" s="6"/>
       <c r="L146" s="6"/>
@@ -10629,8 +10629,8 @@
       <c r="E147" s="6"/>
       <c r="F147" s="6"/>
       <c r="G147" s="6"/>
-      <c r="H147" s="315"/>
-      <c r="I147" s="317"/>
+      <c r="H147" s="313"/>
+      <c r="I147" s="315"/>
       <c r="J147" s="6"/>
       <c r="K147" s="6"/>
       <c r="L147" s="6"/>
@@ -10664,8 +10664,8 @@
       <c r="E148" s="6"/>
       <c r="F148" s="6"/>
       <c r="G148" s="6"/>
-      <c r="H148" s="315"/>
-      <c r="I148" s="317"/>
+      <c r="H148" s="313"/>
+      <c r="I148" s="315"/>
       <c r="J148" s="6"/>
       <c r="K148" s="6"/>
       <c r="L148" s="6"/>
@@ -10699,8 +10699,8 @@
       <c r="E149" s="6"/>
       <c r="F149" s="6"/>
       <c r="G149" s="6"/>
-      <c r="H149" s="315"/>
-      <c r="I149" s="317"/>
+      <c r="H149" s="313"/>
+      <c r="I149" s="315"/>
       <c r="J149" s="6"/>
       <c r="K149" s="6"/>
       <c r="L149" s="6"/>
@@ -10734,8 +10734,8 @@
       <c r="E150" s="6"/>
       <c r="F150" s="6"/>
       <c r="G150" s="6"/>
-      <c r="H150" s="315"/>
-      <c r="I150" s="317"/>
+      <c r="H150" s="313"/>
+      <c r="I150" s="315"/>
       <c r="J150" s="6"/>
       <c r="K150" s="6"/>
       <c r="L150" s="6"/>
@@ -10769,8 +10769,8 @@
       <c r="E151" s="6"/>
       <c r="F151" s="6"/>
       <c r="G151" s="6"/>
-      <c r="H151" s="315"/>
-      <c r="I151" s="317"/>
+      <c r="H151" s="313"/>
+      <c r="I151" s="315"/>
       <c r="J151" s="6"/>
       <c r="K151" s="6"/>
       <c r="L151" s="6"/>
@@ -10804,8 +10804,8 @@
       <c r="E152" s="6"/>
       <c r="F152" s="6"/>
       <c r="G152" s="6"/>
-      <c r="H152" s="315"/>
-      <c r="I152" s="317"/>
+      <c r="H152" s="313"/>
+      <c r="I152" s="315"/>
       <c r="J152" s="6"/>
       <c r="K152" s="6"/>
       <c r="L152" s="6"/>
@@ -10839,8 +10839,8 @@
       <c r="E153" s="6"/>
       <c r="F153" s="6"/>
       <c r="G153" s="6"/>
-      <c r="H153" s="315"/>
-      <c r="I153" s="317"/>
+      <c r="H153" s="313"/>
+      <c r="I153" s="315"/>
       <c r="J153" s="6"/>
       <c r="K153" s="6"/>
       <c r="L153" s="6"/>
@@ -10874,8 +10874,8 @@
       <c r="E154" s="6"/>
       <c r="F154" s="6"/>
       <c r="G154" s="6"/>
-      <c r="H154" s="315"/>
-      <c r="I154" s="317"/>
+      <c r="H154" s="313"/>
+      <c r="I154" s="315"/>
       <c r="J154" s="6"/>
       <c r="K154" s="6"/>
       <c r="L154" s="6"/>
@@ -10909,8 +10909,8 @@
       <c r="E155" s="6"/>
       <c r="F155" s="6"/>
       <c r="G155" s="6"/>
-      <c r="H155" s="315"/>
-      <c r="I155" s="317"/>
+      <c r="H155" s="313"/>
+      <c r="I155" s="315"/>
       <c r="J155" s="6"/>
       <c r="K155" s="6"/>
       <c r="L155" s="6"/>
@@ -10944,8 +10944,8 @@
       <c r="E156" s="6"/>
       <c r="F156" s="6"/>
       <c r="G156" s="6"/>
-      <c r="H156" s="315"/>
-      <c r="I156" s="317"/>
+      <c r="H156" s="313"/>
+      <c r="I156" s="315"/>
       <c r="J156" s="6"/>
       <c r="K156" s="6"/>
       <c r="L156" s="6"/>
@@ -10979,8 +10979,8 @@
       <c r="E157" s="6"/>
       <c r="F157" s="6"/>
       <c r="G157" s="6"/>
-      <c r="H157" s="315"/>
-      <c r="I157" s="317"/>
+      <c r="H157" s="313"/>
+      <c r="I157" s="315"/>
       <c r="J157" s="6"/>
       <c r="K157" s="6"/>
       <c r="L157" s="6"/>
@@ -11014,8 +11014,8 @@
       <c r="E158" s="6"/>
       <c r="F158" s="6"/>
       <c r="G158" s="6"/>
-      <c r="H158" s="315"/>
-      <c r="I158" s="317"/>
+      <c r="H158" s="313"/>
+      <c r="I158" s="315"/>
       <c r="J158" s="6"/>
       <c r="K158" s="6"/>
       <c r="L158" s="6"/>
@@ -11049,8 +11049,8 @@
       <c r="E159" s="6"/>
       <c r="F159" s="6"/>
       <c r="G159" s="6"/>
-      <c r="H159" s="315"/>
-      <c r="I159" s="317"/>
+      <c r="H159" s="313"/>
+      <c r="I159" s="315"/>
       <c r="J159" s="6"/>
       <c r="K159" s="6"/>
       <c r="L159" s="6"/>
@@ -11084,8 +11084,8 @@
       <c r="E160" s="6"/>
       <c r="F160" s="6"/>
       <c r="G160" s="6"/>
-      <c r="H160" s="315"/>
-      <c r="I160" s="317"/>
+      <c r="H160" s="313"/>
+      <c r="I160" s="315"/>
       <c r="J160" s="6"/>
       <c r="K160" s="6"/>
       <c r="L160" s="6"/>
@@ -11119,8 +11119,8 @@
       <c r="E161" s="6"/>
       <c r="F161" s="6"/>
       <c r="G161" s="6"/>
-      <c r="H161" s="315"/>
-      <c r="I161" s="317"/>
+      <c r="H161" s="313"/>
+      <c r="I161" s="315"/>
       <c r="J161" s="6"/>
       <c r="K161" s="6"/>
       <c r="L161" s="6"/>
@@ -11154,8 +11154,8 @@
       <c r="E162" s="6"/>
       <c r="F162" s="6"/>
       <c r="G162" s="6"/>
-      <c r="H162" s="315"/>
-      <c r="I162" s="317"/>
+      <c r="H162" s="313"/>
+      <c r="I162" s="315"/>
       <c r="J162" s="6"/>
       <c r="K162" s="6"/>
       <c r="L162" s="6"/>
@@ -11189,8 +11189,8 @@
       <c r="E163" s="6"/>
       <c r="F163" s="6"/>
       <c r="G163" s="6"/>
-      <c r="H163" s="315"/>
-      <c r="I163" s="317"/>
+      <c r="H163" s="313"/>
+      <c r="I163" s="315"/>
       <c r="J163" s="6"/>
       <c r="K163" s="6"/>
       <c r="L163" s="6"/>
@@ -11224,8 +11224,8 @@
       <c r="E164" s="6"/>
       <c r="F164" s="6"/>
       <c r="G164" s="6"/>
-      <c r="H164" s="315"/>
-      <c r="I164" s="317"/>
+      <c r="H164" s="313"/>
+      <c r="I164" s="315"/>
       <c r="J164" s="6"/>
       <c r="K164" s="6"/>
       <c r="L164" s="6"/>
@@ -11259,8 +11259,8 @@
       <c r="E165" s="6"/>
       <c r="F165" s="6"/>
       <c r="G165" s="6"/>
-      <c r="H165" s="315"/>
-      <c r="I165" s="317"/>
+      <c r="H165" s="313"/>
+      <c r="I165" s="315"/>
       <c r="J165" s="6"/>
       <c r="K165" s="6"/>
       <c r="L165" s="6"/>
@@ -11294,8 +11294,8 @@
       <c r="E166" s="6"/>
       <c r="F166" s="6"/>
       <c r="G166" s="6"/>
-      <c r="H166" s="315"/>
-      <c r="I166" s="317"/>
+      <c r="H166" s="313"/>
+      <c r="I166" s="315"/>
       <c r="J166" s="6"/>
       <c r="K166" s="6"/>
       <c r="L166" s="6"/>
@@ -11329,8 +11329,8 @@
       <c r="E167" s="6"/>
       <c r="F167" s="6"/>
       <c r="G167" s="6"/>
-      <c r="H167" s="315"/>
-      <c r="I167" s="317"/>
+      <c r="H167" s="313"/>
+      <c r="I167" s="315"/>
       <c r="J167" s="6"/>
       <c r="K167" s="6"/>
       <c r="L167" s="6"/>
@@ -11364,8 +11364,8 @@
       <c r="E168" s="6"/>
       <c r="F168" s="6"/>
       <c r="G168" s="6"/>
-      <c r="H168" s="315"/>
-      <c r="I168" s="317"/>
+      <c r="H168" s="313"/>
+      <c r="I168" s="315"/>
       <c r="J168" s="6"/>
       <c r="K168" s="6"/>
       <c r="L168" s="6"/>
@@ -11399,8 +11399,8 @@
       <c r="E169" s="6"/>
       <c r="F169" s="6"/>
       <c r="G169" s="6"/>
-      <c r="H169" s="315"/>
-      <c r="I169" s="317"/>
+      <c r="H169" s="313"/>
+      <c r="I169" s="315"/>
       <c r="J169" s="6"/>
       <c r="K169" s="6"/>
       <c r="L169" s="6"/>
@@ -11434,8 +11434,8 @@
       <c r="E170" s="6"/>
       <c r="F170" s="6"/>
       <c r="G170" s="6"/>
-      <c r="H170" s="315"/>
-      <c r="I170" s="317"/>
+      <c r="H170" s="313"/>
+      <c r="I170" s="315"/>
       <c r="J170" s="6"/>
       <c r="K170" s="6"/>
       <c r="L170" s="6"/>
@@ -11469,8 +11469,8 @@
       <c r="E171" s="6"/>
       <c r="F171" s="6"/>
       <c r="G171" s="6"/>
-      <c r="H171" s="315"/>
-      <c r="I171" s="317"/>
+      <c r="H171" s="313"/>
+      <c r="I171" s="315"/>
       <c r="J171" s="6"/>
       <c r="K171" s="6"/>
       <c r="L171" s="6"/>
@@ -11504,8 +11504,8 @@
       <c r="E172" s="6"/>
       <c r="F172" s="6"/>
       <c r="G172" s="6"/>
-      <c r="H172" s="315"/>
-      <c r="I172" s="317"/>
+      <c r="H172" s="313"/>
+      <c r="I172" s="315"/>
       <c r="J172" s="6"/>
       <c r="K172" s="6"/>
       <c r="L172" s="6"/>
@@ -11539,8 +11539,8 @@
       <c r="E173" s="6"/>
       <c r="F173" s="6"/>
       <c r="G173" s="6"/>
-      <c r="H173" s="315"/>
-      <c r="I173" s="317"/>
+      <c r="H173" s="313"/>
+      <c r="I173" s="315"/>
       <c r="J173" s="6"/>
       <c r="K173" s="6"/>
       <c r="L173" s="6"/>
@@ -11574,8 +11574,8 @@
       <c r="E174" s="6"/>
       <c r="F174" s="6"/>
       <c r="G174" s="6"/>
-      <c r="H174" s="315"/>
-      <c r="I174" s="317"/>
+      <c r="H174" s="313"/>
+      <c r="I174" s="315"/>
       <c r="J174" s="6"/>
       <c r="K174" s="6"/>
       <c r="L174" s="6"/>
@@ -11609,8 +11609,8 @@
       <c r="E175" s="6"/>
       <c r="F175" s="6"/>
       <c r="G175" s="6"/>
-      <c r="H175" s="315"/>
-      <c r="I175" s="317"/>
+      <c r="H175" s="313"/>
+      <c r="I175" s="315"/>
       <c r="J175" s="6"/>
       <c r="K175" s="6"/>
       <c r="L175" s="6"/>
@@ -11644,8 +11644,8 @@
       <c r="E176" s="6"/>
       <c r="F176" s="6"/>
       <c r="G176" s="6"/>
-      <c r="H176" s="315"/>
-      <c r="I176" s="317"/>
+      <c r="H176" s="313"/>
+      <c r="I176" s="315"/>
       <c r="J176" s="6"/>
       <c r="K176" s="6"/>
       <c r="L176" s="6"/>
@@ -11679,8 +11679,8 @@
       <c r="E177" s="6"/>
       <c r="F177" s="6"/>
       <c r="G177" s="6"/>
-      <c r="H177" s="315"/>
-      <c r="I177" s="317"/>
+      <c r="H177" s="313"/>
+      <c r="I177" s="315"/>
       <c r="J177" s="6"/>
       <c r="K177" s="6"/>
       <c r="L177" s="6"/>
@@ -11714,8 +11714,8 @@
       <c r="E178" s="6"/>
       <c r="F178" s="6"/>
       <c r="G178" s="6"/>
-      <c r="H178" s="315"/>
-      <c r="I178" s="317"/>
+      <c r="H178" s="313"/>
+      <c r="I178" s="315"/>
       <c r="J178" s="6"/>
       <c r="K178" s="6"/>
       <c r="L178" s="6"/>
@@ -11749,8 +11749,8 @@
       <c r="E179" s="6"/>
       <c r="F179" s="6"/>
       <c r="G179" s="6"/>
-      <c r="H179" s="315"/>
-      <c r="I179" s="317"/>
+      <c r="H179" s="313"/>
+      <c r="I179" s="315"/>
       <c r="J179" s="6"/>
       <c r="K179" s="6"/>
       <c r="L179" s="6"/>
@@ -11784,8 +11784,8 @@
       <c r="E180" s="6"/>
       <c r="F180" s="6"/>
       <c r="G180" s="6"/>
-      <c r="H180" s="315"/>
-      <c r="I180" s="317"/>
+      <c r="H180" s="313"/>
+      <c r="I180" s="315"/>
       <c r="J180" s="6"/>
       <c r="K180" s="6"/>
       <c r="L180" s="6"/>
@@ -11819,8 +11819,8 @@
       <c r="E181" s="6"/>
       <c r="F181" s="6"/>
       <c r="G181" s="6"/>
-      <c r="H181" s="315"/>
-      <c r="I181" s="317"/>
+      <c r="H181" s="313"/>
+      <c r="I181" s="315"/>
       <c r="J181" s="6"/>
       <c r="K181" s="6"/>
       <c r="L181" s="6"/>
@@ -11854,8 +11854,8 @@
       <c r="E182" s="6"/>
       <c r="F182" s="6"/>
       <c r="G182" s="6"/>
-      <c r="H182" s="315"/>
-      <c r="I182" s="317"/>
+      <c r="H182" s="313"/>
+      <c r="I182" s="315"/>
       <c r="J182" s="6"/>
       <c r="K182" s="6"/>
       <c r="L182" s="6"/>
@@ -11889,8 +11889,8 @@
       <c r="E183" s="6"/>
       <c r="F183" s="6"/>
       <c r="G183" s="6"/>
-      <c r="H183" s="315"/>
-      <c r="I183" s="317"/>
+      <c r="H183" s="313"/>
+      <c r="I183" s="315"/>
       <c r="J183" s="6"/>
       <c r="K183" s="6"/>
       <c r="L183" s="6"/>
@@ -11924,8 +11924,8 @@
       <c r="E184" s="6"/>
       <c r="F184" s="6"/>
       <c r="G184" s="6"/>
-      <c r="H184" s="315"/>
-      <c r="I184" s="317"/>
+      <c r="H184" s="313"/>
+      <c r="I184" s="315"/>
       <c r="J184" s="6"/>
       <c r="K184" s="6"/>
       <c r="L184" s="6"/>
@@ -11959,8 +11959,8 @@
       <c r="E185" s="6"/>
       <c r="F185" s="6"/>
       <c r="G185" s="6"/>
-      <c r="H185" s="315"/>
-      <c r="I185" s="317"/>
+      <c r="H185" s="313"/>
+      <c r="I185" s="315"/>
       <c r="J185" s="6"/>
       <c r="K185" s="6"/>
       <c r="L185" s="6"/>
@@ -11994,8 +11994,8 @@
       <c r="E186" s="6"/>
       <c r="F186" s="6"/>
       <c r="G186" s="6"/>
-      <c r="H186" s="315"/>
-      <c r="I186" s="317"/>
+      <c r="H186" s="313"/>
+      <c r="I186" s="315"/>
       <c r="J186" s="6"/>
       <c r="K186" s="6"/>
       <c r="L186" s="6"/>
@@ -12029,8 +12029,8 @@
       <c r="E187" s="6"/>
       <c r="F187" s="6"/>
       <c r="G187" s="6"/>
-      <c r="H187" s="315"/>
-      <c r="I187" s="317"/>
+      <c r="H187" s="313"/>
+      <c r="I187" s="315"/>
       <c r="J187" s="6"/>
       <c r="K187" s="6"/>
       <c r="L187" s="6"/>
@@ -12064,8 +12064,8 @@
       <c r="E188" s="6"/>
       <c r="F188" s="6"/>
       <c r="G188" s="6"/>
-      <c r="H188" s="315"/>
-      <c r="I188" s="317"/>
+      <c r="H188" s="313"/>
+      <c r="I188" s="315"/>
       <c r="J188" s="6"/>
       <c r="K188" s="6"/>
       <c r="L188" s="6"/>
@@ -12099,8 +12099,8 @@
       <c r="E189" s="6"/>
       <c r="F189" s="6"/>
       <c r="G189" s="6"/>
-      <c r="H189" s="315"/>
-      <c r="I189" s="317"/>
+      <c r="H189" s="313"/>
+      <c r="I189" s="315"/>
       <c r="J189" s="6"/>
       <c r="K189" s="6"/>
       <c r="L189" s="6"/>
@@ -12134,8 +12134,8 @@
       <c r="E190" s="6"/>
       <c r="F190" s="6"/>
       <c r="G190" s="6"/>
-      <c r="H190" s="315"/>
-      <c r="I190" s="317"/>
+      <c r="H190" s="313"/>
+      <c r="I190" s="315"/>
       <c r="J190" s="6"/>
       <c r="K190" s="6"/>
       <c r="L190" s="6"/>
@@ -12169,8 +12169,8 @@
       <c r="E191" s="6"/>
       <c r="F191" s="6"/>
       <c r="G191" s="6"/>
-      <c r="H191" s="315"/>
-      <c r="I191" s="317"/>
+      <c r="H191" s="313"/>
+      <c r="I191" s="315"/>
       <c r="J191" s="6"/>
       <c r="K191" s="6"/>
       <c r="L191" s="6"/>
@@ -12204,8 +12204,8 @@
       <c r="E192" s="6"/>
       <c r="F192" s="6"/>
       <c r="G192" s="6"/>
-      <c r="H192" s="315"/>
-      <c r="I192" s="317"/>
+      <c r="H192" s="313"/>
+      <c r="I192" s="315"/>
       <c r="J192" s="6"/>
       <c r="K192" s="6"/>
       <c r="L192" s="6"/>
@@ -12239,8 +12239,8 @@
       <c r="E193" s="6"/>
       <c r="F193" s="6"/>
       <c r="G193" s="6"/>
-      <c r="H193" s="315"/>
-      <c r="I193" s="317"/>
+      <c r="H193" s="313"/>
+      <c r="I193" s="315"/>
       <c r="J193" s="6"/>
       <c r="K193" s="6"/>
       <c r="L193" s="6"/>
@@ -12274,8 +12274,8 @@
       <c r="E194" s="6"/>
       <c r="F194" s="6"/>
       <c r="G194" s="6"/>
-      <c r="H194" s="315"/>
-      <c r="I194" s="317"/>
+      <c r="H194" s="313"/>
+      <c r="I194" s="315"/>
       <c r="J194" s="6"/>
       <c r="K194" s="6"/>
       <c r="L194" s="6"/>
@@ -12309,8 +12309,8 @@
       <c r="E195" s="6"/>
       <c r="F195" s="6"/>
       <c r="G195" s="6"/>
-      <c r="H195" s="315"/>
-      <c r="I195" s="317"/>
+      <c r="H195" s="313"/>
+      <c r="I195" s="315"/>
       <c r="J195" s="6"/>
       <c r="K195" s="6"/>
       <c r="L195" s="6"/>
@@ -12344,8 +12344,8 @@
       <c r="E196" s="6"/>
       <c r="F196" s="6"/>
       <c r="G196" s="6"/>
-      <c r="H196" s="315"/>
-      <c r="I196" s="317"/>
+      <c r="H196" s="313"/>
+      <c r="I196" s="315"/>
       <c r="J196" s="6"/>
       <c r="K196" s="6"/>
       <c r="L196" s="6"/>
@@ -12379,8 +12379,8 @@
       <c r="E197" s="6"/>
       <c r="F197" s="6"/>
       <c r="G197" s="6"/>
-      <c r="H197" s="315"/>
-      <c r="I197" s="317"/>
+      <c r="H197" s="313"/>
+      <c r="I197" s="315"/>
       <c r="J197" s="6"/>
       <c r="K197" s="6"/>
       <c r="L197" s="6"/>
@@ -12414,8 +12414,8 @@
       <c r="E198" s="6"/>
       <c r="F198" s="6"/>
       <c r="G198" s="6"/>
-      <c r="H198" s="315"/>
-      <c r="I198" s="317"/>
+      <c r="H198" s="313"/>
+      <c r="I198" s="315"/>
       <c r="J198" s="6"/>
       <c r="K198" s="6"/>
       <c r="L198" s="6"/>
@@ -12449,8 +12449,8 @@
       <c r="E199" s="6"/>
       <c r="F199" s="6"/>
       <c r="G199" s="6"/>
-      <c r="H199" s="315"/>
-      <c r="I199" s="317"/>
+      <c r="H199" s="313"/>
+      <c r="I199" s="315"/>
       <c r="J199" s="6"/>
       <c r="K199" s="6"/>
       <c r="L199" s="6"/>
@@ -12484,8 +12484,8 @@
       <c r="E200" s="6"/>
       <c r="F200" s="6"/>
       <c r="G200" s="6"/>
-      <c r="H200" s="315"/>
-      <c r="I200" s="317"/>
+      <c r="H200" s="313"/>
+      <c r="I200" s="315"/>
       <c r="J200" s="6"/>
       <c r="K200" s="6"/>
       <c r="L200" s="6"/>
@@ -12519,8 +12519,8 @@
       <c r="E201" s="6"/>
       <c r="F201" s="6"/>
       <c r="G201" s="6"/>
-      <c r="H201" s="315"/>
-      <c r="I201" s="317"/>
+      <c r="H201" s="313"/>
+      <c r="I201" s="315"/>
       <c r="J201" s="6"/>
       <c r="K201" s="6"/>
       <c r="L201" s="6"/>
@@ -12554,8 +12554,8 @@
       <c r="E202" s="6"/>
       <c r="F202" s="6"/>
       <c r="G202" s="6"/>
-      <c r="H202" s="315"/>
-      <c r="I202" s="317"/>
+      <c r="H202" s="313"/>
+      <c r="I202" s="315"/>
       <c r="J202" s="6"/>
       <c r="K202" s="6"/>
       <c r="L202" s="6"/>
@@ -12589,8 +12589,8 @@
       <c r="E203" s="6"/>
       <c r="F203" s="6"/>
       <c r="G203" s="6"/>
-      <c r="H203" s="315"/>
-      <c r="I203" s="317"/>
+      <c r="H203" s="313"/>
+      <c r="I203" s="315"/>
       <c r="J203" s="6"/>
       <c r="K203" s="6"/>
       <c r="L203" s="6"/>
@@ -12624,8 +12624,8 @@
       <c r="E204" s="6"/>
       <c r="F204" s="6"/>
       <c r="G204" s="6"/>
-      <c r="H204" s="315"/>
-      <c r="I204" s="317"/>
+      <c r="H204" s="313"/>
+      <c r="I204" s="315"/>
       <c r="J204" s="6"/>
       <c r="K204" s="6"/>
       <c r="L204" s="6"/>
@@ -12659,8 +12659,8 @@
       <c r="E205" s="6"/>
       <c r="F205" s="6"/>
       <c r="G205" s="6"/>
-      <c r="H205" s="315"/>
-      <c r="I205" s="317"/>
+      <c r="H205" s="313"/>
+      <c r="I205" s="315"/>
       <c r="J205" s="6"/>
       <c r="K205" s="6"/>
       <c r="L205" s="6"/>
@@ -12694,8 +12694,8 @@
       <c r="E206" s="6"/>
       <c r="F206" s="6"/>
       <c r="G206" s="6"/>
-      <c r="H206" s="315"/>
-      <c r="I206" s="317"/>
+      <c r="H206" s="313"/>
+      <c r="I206" s="315"/>
       <c r="J206" s="6"/>
       <c r="K206" s="6"/>
       <c r="L206" s="6"/>
@@ -12729,8 +12729,8 @@
       <c r="E207" s="6"/>
       <c r="F207" s="6"/>
       <c r="G207" s="6"/>
-      <c r="H207" s="315"/>
-      <c r="I207" s="317"/>
+      <c r="H207" s="313"/>
+      <c r="I207" s="315"/>
       <c r="J207" s="6"/>
       <c r="K207" s="6"/>
       <c r="L207" s="6"/>
@@ -12764,8 +12764,8 @@
       <c r="E208" s="6"/>
       <c r="F208" s="6"/>
       <c r="G208" s="6"/>
-      <c r="H208" s="315"/>
-      <c r="I208" s="317"/>
+      <c r="H208" s="313"/>
+      <c r="I208" s="315"/>
       <c r="J208" s="6"/>
       <c r="K208" s="6"/>
       <c r="L208" s="6"/>
@@ -12799,8 +12799,8 @@
       <c r="E209" s="6"/>
       <c r="F209" s="6"/>
       <c r="G209" s="6"/>
-      <c r="H209" s="315"/>
-      <c r="I209" s="317"/>
+      <c r="H209" s="313"/>
+      <c r="I209" s="315"/>
       <c r="J209" s="6"/>
       <c r="K209" s="6"/>
       <c r="L209" s="6"/>
@@ -12834,8 +12834,8 @@
       <c r="E210" s="6"/>
       <c r="F210" s="6"/>
       <c r="G210" s="6"/>
-      <c r="H210" s="315"/>
-      <c r="I210" s="317"/>
+      <c r="H210" s="313"/>
+      <c r="I210" s="315"/>
       <c r="J210" s="6"/>
       <c r="K210" s="6"/>
       <c r="L210" s="6"/>
@@ -12869,8 +12869,8 @@
       <c r="E211" s="6"/>
       <c r="F211" s="6"/>
       <c r="G211" s="6"/>
-      <c r="H211" s="315"/>
-      <c r="I211" s="317"/>
+      <c r="H211" s="313"/>
+      <c r="I211" s="315"/>
       <c r="J211" s="6"/>
       <c r="K211" s="6"/>
       <c r="L211" s="6"/>
@@ -12904,8 +12904,8 @@
       <c r="E212" s="6"/>
       <c r="F212" s="6"/>
       <c r="G212" s="6"/>
-      <c r="H212" s="315"/>
-      <c r="I212" s="317"/>
+      <c r="H212" s="313"/>
+      <c r="I212" s="315"/>
       <c r="J212" s="6"/>
       <c r="K212" s="6"/>
       <c r="L212" s="6"/>
@@ -12939,8 +12939,8 @@
       <c r="E213" s="6"/>
       <c r="F213" s="6"/>
       <c r="G213" s="6"/>
-      <c r="H213" s="315"/>
-      <c r="I213" s="317"/>
+      <c r="H213" s="313"/>
+      <c r="I213" s="315"/>
       <c r="J213" s="6"/>
       <c r="K213" s="6"/>
       <c r="L213" s="6"/>
@@ -12974,8 +12974,8 @@
       <c r="E214" s="6"/>
       <c r="F214" s="6"/>
       <c r="G214" s="6"/>
-      <c r="H214" s="315"/>
-      <c r="I214" s="317"/>
+      <c r="H214" s="313"/>
+      <c r="I214" s="315"/>
       <c r="J214" s="6"/>
       <c r="K214" s="6"/>
       <c r="L214" s="6"/>
@@ -13009,8 +13009,8 @@
       <c r="E215" s="6"/>
       <c r="F215" s="6"/>
       <c r="G215" s="6"/>
-      <c r="H215" s="315"/>
-      <c r="I215" s="317"/>
+      <c r="H215" s="313"/>
+      <c r="I215" s="315"/>
       <c r="J215" s="6"/>
       <c r="K215" s="6"/>
       <c r="L215" s="6"/>
@@ -13044,8 +13044,8 @@
       <c r="E216" s="6"/>
       <c r="F216" s="6"/>
       <c r="G216" s="6"/>
-      <c r="H216" s="315"/>
-      <c r="I216" s="317"/>
+      <c r="H216" s="313"/>
+      <c r="I216" s="315"/>
       <c r="J216" s="6"/>
       <c r="K216" s="6"/>
       <c r="L216" s="6"/>
@@ -13079,8 +13079,8 @@
       <c r="E217" s="6"/>
       <c r="F217" s="6"/>
       <c r="G217" s="6"/>
-      <c r="H217" s="315"/>
-      <c r="I217" s="317"/>
+      <c r="H217" s="313"/>
+      <c r="I217" s="315"/>
       <c r="J217" s="6"/>
       <c r="K217" s="6"/>
       <c r="L217" s="6"/>
@@ -13114,8 +13114,8 @@
       <c r="E218" s="6"/>
       <c r="F218" s="6"/>
       <c r="G218" s="6"/>
-      <c r="H218" s="315"/>
-      <c r="I218" s="317"/>
+      <c r="H218" s="313"/>
+      <c r="I218" s="315"/>
       <c r="J218" s="6"/>
       <c r="K218" s="6"/>
       <c r="L218" s="6"/>
@@ -13149,8 +13149,8 @@
       <c r="E219" s="6"/>
       <c r="F219" s="6"/>
       <c r="G219" s="6"/>
-      <c r="H219" s="315"/>
-      <c r="I219" s="317"/>
+      <c r="H219" s="313"/>
+      <c r="I219" s="315"/>
       <c r="J219" s="6"/>
       <c r="K219" s="6"/>
       <c r="L219" s="6"/>
@@ -13184,8 +13184,8 @@
       <c r="E220" s="6"/>
       <c r="F220" s="6"/>
       <c r="G220" s="6"/>
-      <c r="H220" s="315"/>
-      <c r="I220" s="317"/>
+      <c r="H220" s="313"/>
+      <c r="I220" s="315"/>
       <c r="J220" s="6"/>
       <c r="K220" s="6"/>
       <c r="L220" s="6"/>
@@ -13219,8 +13219,8 @@
       <c r="E221" s="6"/>
       <c r="F221" s="6"/>
       <c r="G221" s="6"/>
-      <c r="H221" s="315"/>
-      <c r="I221" s="317"/>
+      <c r="H221" s="313"/>
+      <c r="I221" s="315"/>
       <c r="J221" s="6"/>
       <c r="K221" s="6"/>
       <c r="L221" s="6"/>
@@ -13254,8 +13254,8 @@
       <c r="E222" s="6"/>
       <c r="F222" s="6"/>
       <c r="G222" s="6"/>
-      <c r="H222" s="315"/>
-      <c r="I222" s="317"/>
+      <c r="H222" s="313"/>
+      <c r="I222" s="315"/>
       <c r="J222" s="6"/>
       <c r="K222" s="6"/>
       <c r="L222" s="6"/>
@@ -13289,8 +13289,8 @@
       <c r="E223" s="6"/>
       <c r="F223" s="6"/>
       <c r="G223" s="6"/>
-      <c r="H223" s="315"/>
-      <c r="I223" s="317"/>
+      <c r="H223" s="313"/>
+      <c r="I223" s="315"/>
       <c r="J223" s="6"/>
       <c r="K223" s="6"/>
       <c r="L223" s="6"/>
@@ -13324,8 +13324,8 @@
       <c r="E224" s="6"/>
       <c r="F224" s="6"/>
       <c r="G224" s="6"/>
-      <c r="H224" s="315"/>
-      <c r="I224" s="317"/>
+      <c r="H224" s="313"/>
+      <c r="I224" s="315"/>
       <c r="J224" s="6"/>
       <c r="K224" s="6"/>
       <c r="L224" s="6"/>
@@ -13493,7 +13493,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50F898A0-50DC-4248-B4D3-1E1F1C494B94}">
   <dimension ref="A1:F9"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="17.7109375" customWidth="1"/>
     <col min="2" max="2" width="23.42578125" customWidth="1"/>
@@ -13619,7 +13619,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EB265A1-AA32-451B-ADDB-D29D34FAE070}">
   <dimension ref="A1:AT252"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18.28515625" customWidth="1"/>
     <col min="2" max="2" width="17.28515625" customWidth="1"/>
@@ -13689,19 +13689,19 @@
       <c r="S1" s="9"/>
       <c r="T1" s="9"/>
       <c r="U1" s="9"/>
-      <c r="V1" s="313" t="s">
+      <c r="V1" s="320" t="s">
         <v>387</v>
       </c>
-      <c r="W1" s="313"/>
-      <c r="X1" s="313"/>
-      <c r="Y1" s="313"/>
-      <c r="Z1" s="313"/>
-      <c r="AA1" s="313"/>
-      <c r="AB1" s="313"/>
-      <c r="AC1" s="313"/>
-      <c r="AD1" s="313"/>
-      <c r="AE1" s="313"/>
-      <c r="AF1" s="314"/>
+      <c r="W1" s="320"/>
+      <c r="X1" s="320"/>
+      <c r="Y1" s="320"/>
+      <c r="Z1" s="320"/>
+      <c r="AA1" s="320"/>
+      <c r="AB1" s="320"/>
+      <c r="AC1" s="320"/>
+      <c r="AD1" s="320"/>
+      <c r="AE1" s="320"/>
+      <c r="AF1" s="321"/>
       <c r="AG1" s="145" t="s">
         <v>2</v>
       </c>
@@ -13725,7 +13725,7 @@
       </c>
       <c r="AT1" s="149"/>
     </row>
-    <row r="2" spans="1:46" s="152" customFormat="1" ht="60.75">
+    <row r="2" spans="1:46" s="152" customFormat="1" ht="60">
       <c r="A2" s="303" t="s">
         <v>388</v>
       </c>
@@ -24419,12 +24419,9 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -24566,19 +24563,45 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{183E6228-D059-4D4A-9844-9FB7E4EC7682}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{695864D4-4D75-4318-98FB-08B4DB48CFF6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9733FB95-B7F1-4430-9D8C-98621A69FCF7}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9733FB95-B7F1-4430-9D8C-98621A69FCF7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="4662f0e3-f4c4-4931-8e76-960ae722852f"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{695864D4-4D75-4318-98FB-08B4DB48CFF6}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{183E6228-D059-4D4A-9844-9FB7E4EC7682}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>